<commit_message>
p502 sync 2026-09-11 10:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2538"/>
+  <dimension ref="A1:D2547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -11266,8 +11266,6 @@
         <v/>
       </c>
     </row>
-    <row r="975"/>
-    <row r="976"/>
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
@@ -11464,7 +11462,6 @@
         <v/>
       </c>
     </row>
-    <row r="996"/>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
@@ -11518,8 +11515,6 @@
         <v/>
       </c>
     </row>
-    <row r="1001"/>
-    <row r="1002"/>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
@@ -11559,8 +11554,6 @@
         <v/>
       </c>
     </row>
-    <row r="1006"/>
-    <row r="1007"/>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
@@ -11682,7 +11675,6 @@
         <v/>
       </c>
     </row>
-    <row r="1019"/>
     <row r="1020">
       <c r="A1020" t="inlineStr">
         <is>
@@ -11736,8 +11728,6 @@
         <v/>
       </c>
     </row>
-    <row r="1024"/>
-    <row r="1025"/>
     <row r="1026">
       <c r="A1026" t="inlineStr">
         <is>
@@ -11777,8 +11767,6 @@
         <v/>
       </c>
     </row>
-    <row r="1029"/>
-    <row r="1030"/>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
@@ -11840,7 +11828,6 @@
         <v/>
       </c>
     </row>
-    <row r="1036"/>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
@@ -11848,7 +11835,6 @@
         </is>
       </c>
     </row>
-    <row r="1038"/>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
@@ -11903,7 +11889,6 @@
         <v/>
       </c>
     </row>
-    <row r="1043"/>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
@@ -11958,7 +11943,6 @@
         <v/>
       </c>
     </row>
-    <row r="1048"/>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
@@ -12080,7 +12064,6 @@
         <v/>
       </c>
     </row>
-    <row r="1060"/>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
@@ -12134,8 +12117,6 @@
         <v/>
       </c>
     </row>
-    <row r="1065"/>
-    <row r="1066"/>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
@@ -12266,7 +12247,6 @@
         <v/>
       </c>
     </row>
-    <row r="1079"/>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
@@ -12320,7 +12300,6 @@
         <v/>
       </c>
     </row>
-    <row r="1084"/>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
@@ -12343,8 +12322,6 @@
         <v>-75037.94</v>
       </c>
     </row>
-    <row r="1087"/>
-    <row r="1088"/>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
@@ -12496,7 +12473,6 @@
         <v/>
       </c>
     </row>
-    <row r="1103"/>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
@@ -12550,7 +12526,6 @@
         <v/>
       </c>
     </row>
-    <row r="1108"/>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
@@ -12604,8 +12579,6 @@
         <v/>
       </c>
     </row>
-    <row r="1113"/>
-    <row r="1114"/>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
@@ -12706,7 +12679,6 @@
         <v/>
       </c>
     </row>
-    <row r="1124"/>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
@@ -12760,8 +12732,6 @@
         <v/>
       </c>
     </row>
-    <row r="1129"/>
-    <row r="1130"/>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
@@ -12925,7 +12895,6 @@
         <v/>
       </c>
     </row>
-    <row r="1146"/>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
@@ -12979,8 +12948,6 @@
         <v/>
       </c>
     </row>
-    <row r="1151"/>
-    <row r="1152"/>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
@@ -13144,7 +13111,6 @@
         <v/>
       </c>
     </row>
-    <row r="1168"/>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
@@ -13198,8 +13164,6 @@
         <v/>
       </c>
     </row>
-    <row r="1173"/>
-    <row r="1174"/>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
@@ -13369,7 +13333,6 @@
         <v/>
       </c>
     </row>
-    <row r="1191"/>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
@@ -13423,7 +13386,6 @@
         <v/>
       </c>
     </row>
-    <row r="1196"/>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
@@ -13476,8 +13438,6 @@
         <v>-74653</v>
       </c>
     </row>
-    <row r="1201"/>
-    <row r="1202"/>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
@@ -13608,7 +13568,6 @@
         <v/>
       </c>
     </row>
-    <row r="1215"/>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
@@ -13662,7 +13621,6 @@
         <v/>
       </c>
     </row>
-    <row r="1220"/>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
@@ -13716,7 +13674,6 @@
         <v/>
       </c>
     </row>
-    <row r="1225"/>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
@@ -13756,8 +13713,6 @@
         <v/>
       </c>
     </row>
-    <row r="1229"/>
-    <row r="1230"/>
     <row r="1231">
       <c r="A1231" s="80" t="inlineStr">
         <is>
@@ -14089,7 +14044,6 @@
         <v/>
       </c>
     </row>
-    <row r="1261"/>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
@@ -14143,7 +14097,6 @@
         <v/>
       </c>
     </row>
-    <row r="1266"/>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
@@ -14198,8 +14151,6 @@
         <v>-74291.5</v>
       </c>
     </row>
-    <row r="1271"/>
-    <row r="1272"/>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
@@ -14531,7 +14482,6 @@
         <v/>
       </c>
     </row>
-    <row r="1305"/>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
@@ -14585,7 +14535,6 @@
         <v/>
       </c>
     </row>
-    <row r="1310"/>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
@@ -14641,8 +14590,6 @@
         <v/>
       </c>
     </row>
-    <row r="1315"/>
-    <row r="1316"/>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
@@ -14878,7 +14825,6 @@
         <v/>
       </c>
     </row>
-    <row r="1339"/>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
@@ -14932,7 +14878,6 @@
         <v/>
       </c>
     </row>
-    <row r="1344"/>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
@@ -15003,7 +14948,6 @@
         <v>-72794.59</v>
       </c>
     </row>
-    <row r="1350"/>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
@@ -15188,7 +15132,6 @@
         <v/>
       </c>
     </row>
-    <row r="1368"/>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
@@ -15242,7 +15185,6 @@
         <v/>
       </c>
     </row>
-    <row r="1373"/>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
@@ -15314,7 +15256,6 @@
         <v/>
       </c>
     </row>
-    <row r="1379"/>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
@@ -15430,7 +15371,6 @@
         <v/>
       </c>
     </row>
-    <row r="1391"/>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
@@ -15484,7 +15424,6 @@
         <v/>
       </c>
     </row>
-    <row r="1396"/>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
@@ -15534,7 +15473,6 @@
         <v/>
       </c>
     </row>
-    <row r="1401"/>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
@@ -15584,7 +15522,6 @@
         <v/>
       </c>
     </row>
-    <row r="1406"/>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
@@ -15634,7 +15571,6 @@
         <v/>
       </c>
     </row>
-    <row r="1411"/>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
@@ -15684,8 +15620,6 @@
         <v/>
       </c>
     </row>
-    <row r="1416"/>
-    <row r="1417"/>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
@@ -15858,7 +15792,6 @@
         <v/>
       </c>
     </row>
-    <row r="1434"/>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
@@ -15915,7 +15848,6 @@
         <v/>
       </c>
     </row>
-    <row r="1439"/>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
@@ -15938,7 +15870,6 @@
         <v>-75313</v>
       </c>
     </row>
-    <row r="1442"/>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
@@ -16291,7 +16222,6 @@
         <v/>
       </c>
     </row>
-    <row r="1476"/>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
@@ -16345,8 +16275,6 @@
         <v/>
       </c>
     </row>
-    <row r="1481"/>
-    <row r="1482"/>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
@@ -16552,7 +16480,6 @@
         <v/>
       </c>
     </row>
-    <row r="1502"/>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
@@ -16606,8 +16533,6 @@
         <v/>
       </c>
     </row>
-    <row r="1507"/>
-    <row r="1508"/>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
@@ -16792,7 +16717,6 @@
         <v/>
       </c>
     </row>
-    <row r="1526"/>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
@@ -16846,8 +16770,6 @@
         <v/>
       </c>
     </row>
-    <row r="1531"/>
-    <row r="1532"/>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
@@ -17053,7 +16975,6 @@
         <v/>
       </c>
     </row>
-    <row r="1552"/>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
@@ -17107,8 +17028,6 @@
         <v/>
       </c>
     </row>
-    <row r="1557"/>
-    <row r="1558"/>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
@@ -17398,7 +17317,6 @@
         <v/>
       </c>
     </row>
-    <row r="1586"/>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
@@ -17452,7 +17370,6 @@
         <v/>
       </c>
     </row>
-    <row r="1591"/>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
@@ -17506,8 +17423,6 @@
         <v/>
       </c>
     </row>
-    <row r="1596"/>
-    <row r="1597"/>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
@@ -17671,7 +17586,6 @@
         <v/>
       </c>
     </row>
-    <row r="1613"/>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
@@ -17725,8 +17639,6 @@
         <v/>
       </c>
     </row>
-    <row r="1618"/>
-    <row r="1619"/>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
@@ -17995,7 +17907,6 @@
         <v/>
       </c>
     </row>
-    <row r="1645"/>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
@@ -18049,8 +17960,6 @@
         <v/>
       </c>
     </row>
-    <row r="1650"/>
-    <row r="1651"/>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
@@ -18277,7 +18186,6 @@
         <v/>
       </c>
     </row>
-    <row r="1673"/>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
@@ -18331,8 +18239,6 @@
         <v/>
       </c>
     </row>
-    <row r="1678"/>
-    <row r="1679"/>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
@@ -18496,7 +18402,6 @@
         <v/>
       </c>
     </row>
-    <row r="1695"/>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
@@ -18550,8 +18455,6 @@
         <v/>
       </c>
     </row>
-    <row r="1700"/>
-    <row r="1701"/>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
@@ -18778,7 +18681,6 @@
         <v/>
       </c>
     </row>
-    <row r="1723"/>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
@@ -18832,8 +18734,6 @@
         <v/>
       </c>
     </row>
-    <row r="1728"/>
-    <row r="1729"/>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
@@ -19291,7 +19191,6 @@
         <v/>
       </c>
     </row>
-    <row r="1773"/>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
@@ -19345,8 +19244,6 @@
         <v/>
       </c>
     </row>
-    <row r="1778"/>
-    <row r="1779"/>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
@@ -19552,7 +19449,6 @@
         <v/>
       </c>
     </row>
-    <row r="1799"/>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
@@ -19606,8 +19502,6 @@
         <v/>
       </c>
     </row>
-    <row r="1804"/>
-    <row r="1805"/>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
@@ -19876,7 +19770,6 @@
         <v/>
       </c>
     </row>
-    <row r="1831"/>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
@@ -19930,8 +19823,6 @@
         <v/>
       </c>
     </row>
-    <row r="1836"/>
-    <row r="1837"/>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
@@ -20158,7 +20049,6 @@
         <v/>
       </c>
     </row>
-    <row r="1859"/>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
@@ -20212,8 +20102,6 @@
         <v/>
       </c>
     </row>
-    <row r="1864"/>
-    <row r="1865"/>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
@@ -20519,7 +20407,6 @@
         <v/>
       </c>
     </row>
-    <row r="1894"/>
     <row r="1895">
       <c r="A1895" t="inlineStr">
         <is>
@@ -20573,7 +20460,6 @@
         <v/>
       </c>
     </row>
-    <row r="1899"/>
     <row r="1900">
       <c r="A1900" t="inlineStr">
         <is>
@@ -20737,7 +20623,6 @@
         <v/>
       </c>
     </row>
-    <row r="1915"/>
     <row r="1916">
       <c r="A1916" t="inlineStr">
         <is>
@@ -21124,8 +21009,6 @@
       </c>
       <c r="D1947" s="40" t="n"/>
     </row>
-    <row r="1948"/>
-    <row r="1949"/>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
@@ -21268,7 +21151,6 @@
         <v/>
       </c>
     </row>
-    <row r="1963"/>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
@@ -21322,8 +21204,6 @@
         <v/>
       </c>
     </row>
-    <row r="1968"/>
-    <row r="1969"/>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
@@ -21508,7 +21388,6 @@
         <v/>
       </c>
     </row>
-    <row r="1987"/>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
@@ -21562,8 +21441,6 @@
         <v/>
       </c>
     </row>
-    <row r="1992"/>
-    <row r="1993"/>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
@@ -22045,7 +21922,6 @@
         <v/>
       </c>
     </row>
-    <row r="2039"/>
     <row r="2040">
       <c r="A2040" t="inlineStr">
         <is>
@@ -22099,7 +21975,6 @@
         <v/>
       </c>
     </row>
-    <row r="2044"/>
     <row r="2045">
       <c r="A2045" t="inlineStr">
         <is>
@@ -22122,8 +21997,6 @@
         <v>-75360.2</v>
       </c>
     </row>
-    <row r="2047"/>
-    <row r="2048"/>
     <row r="2049">
       <c r="A2049" t="inlineStr">
         <is>
@@ -22518,7 +22391,6 @@
         <v/>
       </c>
     </row>
-    <row r="2086"/>
     <row r="2087">
       <c r="A2087" t="inlineStr">
         <is>
@@ -22572,8 +22444,6 @@
         <v/>
       </c>
     </row>
-    <row r="2091"/>
-    <row r="2092"/>
     <row r="2093">
       <c r="A2093" t="inlineStr">
         <is>
@@ -22695,7 +22565,6 @@
         <v/>
       </c>
     </row>
-    <row r="2104"/>
     <row r="2105">
       <c r="A2105" t="inlineStr">
         <is>
@@ -22749,8 +22618,6 @@
         <v/>
       </c>
     </row>
-    <row r="2109"/>
-    <row r="2110"/>
     <row r="2111">
       <c r="A2111" t="inlineStr">
         <is>
@@ -23019,7 +22886,6 @@
         <v/>
       </c>
     </row>
-    <row r="2136"/>
     <row r="2137">
       <c r="A2137" t="inlineStr">
         <is>
@@ -23073,8 +22939,6 @@
         <v/>
       </c>
     </row>
-    <row r="2141"/>
-    <row r="2142"/>
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
@@ -23322,7 +23186,6 @@
         <v/>
       </c>
     </row>
-    <row r="2166"/>
     <row r="2167">
       <c r="A2167" t="inlineStr">
         <is>
@@ -23376,8 +23239,6 @@
         <v/>
       </c>
     </row>
-    <row r="2171"/>
-    <row r="2172"/>
     <row r="2173">
       <c r="A2173" t="inlineStr">
         <is>
@@ -23583,7 +23444,6 @@
         <v/>
       </c>
     </row>
-    <row r="2192"/>
     <row r="2193">
       <c r="A2193" t="inlineStr">
         <is>
@@ -23637,8 +23497,6 @@
         <v/>
       </c>
     </row>
-    <row r="2197"/>
-    <row r="2198"/>
     <row r="2199">
       <c r="A2199" t="inlineStr">
         <is>
@@ -23823,7 +23681,6 @@
         <v/>
       </c>
     </row>
-    <row r="2216"/>
     <row r="2217">
       <c r="A2217" t="inlineStr">
         <is>
@@ -23877,8 +23734,6 @@
         <v/>
       </c>
     </row>
-    <row r="2221"/>
-    <row r="2222"/>
     <row r="2223">
       <c r="A2223" t="inlineStr">
         <is>
@@ -24021,7 +23876,6 @@
         <v/>
       </c>
     </row>
-    <row r="2236"/>
     <row r="2237">
       <c r="A2237" t="inlineStr">
         <is>
@@ -24075,8 +23929,6 @@
         <v/>
       </c>
     </row>
-    <row r="2241"/>
-    <row r="2242"/>
     <row r="2243">
       <c r="A2243" t="inlineStr">
         <is>
@@ -24345,7 +24197,6 @@
         <v/>
       </c>
     </row>
-    <row r="2268"/>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
@@ -24399,8 +24250,6 @@
         <v/>
       </c>
     </row>
-    <row r="2273"/>
-    <row r="2274"/>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
@@ -24711,7 +24560,6 @@
         <v/>
       </c>
     </row>
-    <row r="2304"/>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
@@ -24765,8 +24613,6 @@
         <v/>
       </c>
     </row>
-    <row r="2309"/>
-    <row r="2310"/>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
@@ -24951,7 +24797,6 @@
         <v/>
       </c>
     </row>
-    <row r="2328"/>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
@@ -25005,8 +24850,6 @@
         <v/>
       </c>
     </row>
-    <row r="2333"/>
-    <row r="2334"/>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
@@ -25233,7 +25076,6 @@
         <v/>
       </c>
     </row>
-    <row r="2356"/>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
@@ -25287,7 +25129,6 @@
         <v/>
       </c>
     </row>
-    <row r="2361"/>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
@@ -25311,8 +25152,6 @@
         <v/>
       </c>
     </row>
-    <row r="2364"/>
-    <row r="2365"/>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
@@ -25359,7 +25198,6 @@
         <v/>
       </c>
     </row>
-    <row r="2370"/>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
@@ -25412,8 +25250,6 @@
         <v/>
       </c>
     </row>
-    <row r="2375"/>
-    <row r="2376"/>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
@@ -25577,7 +25413,6 @@
         <v/>
       </c>
     </row>
-    <row r="2392"/>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
@@ -25631,8 +25466,6 @@
         <v/>
       </c>
     </row>
-    <row r="2397"/>
-    <row r="2398"/>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
@@ -25922,7 +25755,6 @@
         <v/>
       </c>
     </row>
-    <row r="2426"/>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
@@ -25976,8 +25808,6 @@
         <v/>
       </c>
     </row>
-    <row r="2431"/>
-    <row r="2432"/>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
@@ -26372,7 +26202,6 @@
         <v/>
       </c>
     </row>
-    <row r="2470"/>
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
@@ -26426,8 +26255,6 @@
         <v/>
       </c>
     </row>
-    <row r="2475"/>
-    <row r="2476"/>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
@@ -26654,7 +26481,6 @@
         <v/>
       </c>
     </row>
-    <row r="2498"/>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
@@ -26708,8 +26534,6 @@
         <v/>
       </c>
     </row>
-    <row r="2503"/>
-    <row r="2504"/>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
@@ -27071,6 +26895,74 @@
       <c r="C2538" s="45">
         <f>C2537/ABS(C2535)</f>
         <v/>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="inlineStr">
+        <is>
+          <t>2026.09.10</t>
+        </is>
+      </c>
+      <c r="B2541" t="n">
+        <v>115848.8</v>
+      </c>
+      <c r="C2541" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" t="n">
+        <v>-75688.5</v>
+      </c>
+      <c r="B2542">
+        <f>+B2541+A2542</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="B2543" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2543">
+        <f>SUM(C2542:C2542)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="B2544" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2544">
+        <f>+B2542-B2541</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" t="inlineStr">
+        <is>
+          <t>累積留倉   100股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="inlineStr">
+        <is>
+          <t>2026.09.10 留倉</t>
+        </is>
+      </c>
+      <c r="B2547" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2547" t="n">
+        <v>-75688.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
p502 sync 2026-09-11 12:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2547"/>
+  <dimension ref="A1:D2556"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -26962,6 +26962,74 @@
         </is>
       </c>
       <c r="C2547" t="n">
+        <v>-75688.5</v>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" t="inlineStr">
+        <is>
+          <t>2026.09.10</t>
+        </is>
+      </c>
+      <c r="B2550" t="n">
+        <v>115848.8</v>
+      </c>
+      <c r="C2550" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="n">
+        <v>-75688.5</v>
+      </c>
+      <c r="B2551">
+        <f>+B2550+A2551</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="B2552" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2552">
+        <f>SUM(C2551:C2551)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="B2553" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2553">
+        <f>+B2551-B2550</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="inlineStr">
+        <is>
+          <t>累積留倉   100股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" t="inlineStr">
+        <is>
+          <t>2026.09.10 留倉</t>
+        </is>
+      </c>
+      <c r="B2556" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2556" t="n">
         <v>-75688.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
p502 sync 2026-09-18 12:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2556"/>
+  <dimension ref="A1:D2571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -27030,6 +27030,139 @@
         </is>
       </c>
       <c r="C2556" t="n">
+        <v>-75688.5</v>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" t="inlineStr">
+        <is>
+          <t>2026.09.16</t>
+        </is>
+      </c>
+      <c r="B2559" t="n">
+        <v>40160.3</v>
+      </c>
+      <c r="C2559" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" t="n">
+        <v>-75916</v>
+      </c>
+      <c r="B2560">
+        <f>+B2559+A2560</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="n">
+        <v>75939.92</v>
+      </c>
+      <c r="B2561">
+        <f>+B2560+A2561</f>
+        <v/>
+      </c>
+      <c r="C2561" t="n">
+        <v>23.92</v>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="B2562" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2562">
+        <f>SUM(C2560:C2561)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="B2563" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2563">
+        <f>+B2561-B2559</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="inlineStr">
+        <is>
+          <t>2026.09.16當沖</t>
+        </is>
+      </c>
+      <c r="B2565" t="inlineStr">
+        <is>
+          <t>買</t>
+        </is>
+      </c>
+      <c r="C2565" s="80">
+        <f>SUMIF(A2560:A2561,"&lt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566">
+        <f>"SPY " &amp; COUNT(C2560:C2561) * 100 &amp; "股"</f>
+        <v/>
+      </c>
+      <c r="B2566" t="inlineStr">
+        <is>
+          <t>賣</t>
+        </is>
+      </c>
+      <c r="C2566" s="80">
+        <f>SUMIF(A2560:A2561,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="B2567" t="inlineStr">
+        <is>
+          <t>當日損益</t>
+        </is>
+      </c>
+      <c r="C2567" s="80">
+        <f>+C2565+C2566</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="B2568" t="inlineStr">
+        <is>
+          <t>當日損益 %</t>
+        </is>
+      </c>
+      <c r="C2568" s="45">
+        <f>C2567/ABS(C2565)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" t="inlineStr">
+        <is>
+          <t>累積留倉   100股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" t="inlineStr">
+        <is>
+          <t>2026.09.10 留倉</t>
+        </is>
+      </c>
+      <c r="B2571" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2571" t="n">
         <v>-75688.5</v>
       </c>
     </row>
@@ -27045,7 +27178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -27835,6 +27968,18 @@
         <v/>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="86" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="C66">
+        <f>C65+B66</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-09-30 13:18
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2584"/>
+  <dimension ref="A1:D2593"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -27215,7 +27215,7 @@
     <row r="2579">
       <c r="A2579" t="inlineStr">
         <is>
-          <t>累積留倉   100股</t>
+          <t>累積留倉   0股</t>
         </is>
       </c>
     </row>
@@ -27286,6 +27286,74 @@
       <c r="C2584" s="42">
         <f>C2583/ABS(C2580)</f>
         <v/>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" t="inlineStr">
+        <is>
+          <t>2026.09.28</t>
+        </is>
+      </c>
+      <c r="B2587" t="n">
+        <v>117089.63</v>
+      </c>
+      <c r="C2587" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2588">
+      <c r="A2588" t="n">
+        <v>-76610.5</v>
+      </c>
+      <c r="B2588">
+        <f>+B2587+A2588</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2589">
+      <c r="B2589" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2589">
+        <f>SUM(C2588:C2588)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2590">
+      <c r="B2590" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2590">
+        <f>+B2588-B2587</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2592">
+      <c r="A2592" t="inlineStr">
+        <is>
+          <t>累積留倉   100股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2593">
+      <c r="A2593" t="inlineStr">
+        <is>
+          <t>2026.09.28 留倉</t>
+        </is>
+      </c>
+      <c r="B2593" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2593" t="n">
+        <v>-76610.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
p502 sync 2026-10-05 18:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2593"/>
+  <dimension ref="A1:E2605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -11266,6 +11266,8 @@
         <v/>
       </c>
     </row>
+    <row r="975"/>
+    <row r="976"/>
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
@@ -11462,6 +11464,7 @@
         <v/>
       </c>
     </row>
+    <row r="996"/>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
@@ -11515,6 +11518,8 @@
         <v/>
       </c>
     </row>
+    <row r="1001"/>
+    <row r="1002"/>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
@@ -11554,6 +11559,8 @@
         <v/>
       </c>
     </row>
+    <row r="1006"/>
+    <row r="1007"/>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
@@ -11675,6 +11682,7 @@
         <v/>
       </c>
     </row>
+    <row r="1019"/>
     <row r="1020">
       <c r="A1020" t="inlineStr">
         <is>
@@ -11728,6 +11736,8 @@
         <v/>
       </c>
     </row>
+    <row r="1024"/>
+    <row r="1025"/>
     <row r="1026">
       <c r="A1026" t="inlineStr">
         <is>
@@ -11767,6 +11777,8 @@
         <v/>
       </c>
     </row>
+    <row r="1029"/>
+    <row r="1030"/>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
@@ -11828,6 +11840,7 @@
         <v/>
       </c>
     </row>
+    <row r="1036"/>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
@@ -11835,6 +11848,7 @@
         </is>
       </c>
     </row>
+    <row r="1038"/>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
@@ -11889,6 +11903,7 @@
         <v/>
       </c>
     </row>
+    <row r="1043"/>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
@@ -11943,6 +11958,7 @@
         <v/>
       </c>
     </row>
+    <row r="1048"/>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
@@ -12064,6 +12080,7 @@
         <v/>
       </c>
     </row>
+    <row r="1060"/>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
@@ -12117,6 +12134,8 @@
         <v/>
       </c>
     </row>
+    <row r="1065"/>
+    <row r="1066"/>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
@@ -12247,6 +12266,7 @@
         <v/>
       </c>
     </row>
+    <row r="1079"/>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
@@ -12300,6 +12320,7 @@
         <v/>
       </c>
     </row>
+    <row r="1084"/>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
@@ -12322,6 +12343,8 @@
         <v>-75037.94</v>
       </c>
     </row>
+    <row r="1087"/>
+    <row r="1088"/>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
@@ -12473,6 +12496,7 @@
         <v/>
       </c>
     </row>
+    <row r="1103"/>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
@@ -12526,6 +12550,7 @@
         <v/>
       </c>
     </row>
+    <row r="1108"/>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
@@ -12579,6 +12604,8 @@
         <v/>
       </c>
     </row>
+    <row r="1113"/>
+    <row r="1114"/>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
@@ -12679,6 +12706,7 @@
         <v/>
       </c>
     </row>
+    <row r="1124"/>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
@@ -12732,6 +12760,8 @@
         <v/>
       </c>
     </row>
+    <row r="1129"/>
+    <row r="1130"/>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
@@ -12895,6 +12925,7 @@
         <v/>
       </c>
     </row>
+    <row r="1146"/>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
@@ -12948,6 +12979,8 @@
         <v/>
       </c>
     </row>
+    <row r="1151"/>
+    <row r="1152"/>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
@@ -13111,6 +13144,7 @@
         <v/>
       </c>
     </row>
+    <row r="1168"/>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
@@ -13164,6 +13198,8 @@
         <v/>
       </c>
     </row>
+    <row r="1173"/>
+    <row r="1174"/>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
@@ -13333,6 +13369,7 @@
         <v/>
       </c>
     </row>
+    <row r="1191"/>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
@@ -13386,6 +13423,7 @@
         <v/>
       </c>
     </row>
+    <row r="1196"/>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
@@ -13438,6 +13476,8 @@
         <v>-74653</v>
       </c>
     </row>
+    <row r="1201"/>
+    <row r="1202"/>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
@@ -13568,6 +13608,7 @@
         <v/>
       </c>
     </row>
+    <row r="1215"/>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
@@ -13621,6 +13662,7 @@
         <v/>
       </c>
     </row>
+    <row r="1220"/>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
@@ -13674,6 +13716,7 @@
         <v/>
       </c>
     </row>
+    <row r="1225"/>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
@@ -13713,6 +13756,8 @@
         <v/>
       </c>
     </row>
+    <row r="1229"/>
+    <row r="1230"/>
     <row r="1231">
       <c r="A1231" s="80" t="inlineStr">
         <is>
@@ -14044,6 +14089,7 @@
         <v/>
       </c>
     </row>
+    <row r="1261"/>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
@@ -14097,6 +14143,7 @@
         <v/>
       </c>
     </row>
+    <row r="1266"/>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
@@ -14151,6 +14198,8 @@
         <v>-74291.5</v>
       </c>
     </row>
+    <row r="1271"/>
+    <row r="1272"/>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
@@ -14482,6 +14531,7 @@
         <v/>
       </c>
     </row>
+    <row r="1305"/>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
@@ -14535,6 +14585,7 @@
         <v/>
       </c>
     </row>
+    <row r="1310"/>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
@@ -14590,6 +14641,8 @@
         <v/>
       </c>
     </row>
+    <row r="1315"/>
+    <row r="1316"/>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
@@ -14825,6 +14878,7 @@
         <v/>
       </c>
     </row>
+    <row r="1339"/>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
@@ -14878,6 +14932,7 @@
         <v/>
       </c>
     </row>
+    <row r="1344"/>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
@@ -14948,6 +15003,7 @@
         <v>-72794.59</v>
       </c>
     </row>
+    <row r="1350"/>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
@@ -15132,6 +15188,7 @@
         <v/>
       </c>
     </row>
+    <row r="1368"/>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
@@ -15185,6 +15242,7 @@
         <v/>
       </c>
     </row>
+    <row r="1373"/>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
@@ -15256,6 +15314,7 @@
         <v/>
       </c>
     </row>
+    <row r="1379"/>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
@@ -15371,6 +15430,7 @@
         <v/>
       </c>
     </row>
+    <row r="1391"/>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
@@ -15424,6 +15484,7 @@
         <v/>
       </c>
     </row>
+    <row r="1396"/>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
@@ -15473,6 +15534,7 @@
         <v/>
       </c>
     </row>
+    <row r="1401"/>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
@@ -15522,6 +15584,7 @@
         <v/>
       </c>
     </row>
+    <row r="1406"/>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
@@ -15571,6 +15634,7 @@
         <v/>
       </c>
     </row>
+    <row r="1411"/>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
@@ -15620,6 +15684,8 @@
         <v/>
       </c>
     </row>
+    <row r="1416"/>
+    <row r="1417"/>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
@@ -15792,6 +15858,7 @@
         <v/>
       </c>
     </row>
+    <row r="1434"/>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
@@ -15848,6 +15915,7 @@
         <v/>
       </c>
     </row>
+    <row r="1439"/>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
@@ -15870,6 +15938,7 @@
         <v>-75313</v>
       </c>
     </row>
+    <row r="1442"/>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
@@ -16222,6 +16291,7 @@
         <v/>
       </c>
     </row>
+    <row r="1476"/>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
@@ -16275,6 +16345,8 @@
         <v/>
       </c>
     </row>
+    <row r="1481"/>
+    <row r="1482"/>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
@@ -16480,6 +16552,7 @@
         <v/>
       </c>
     </row>
+    <row r="1502"/>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
@@ -16533,6 +16606,8 @@
         <v/>
       </c>
     </row>
+    <row r="1507"/>
+    <row r="1508"/>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
@@ -16717,6 +16792,7 @@
         <v/>
       </c>
     </row>
+    <row r="1526"/>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
@@ -16770,6 +16846,8 @@
         <v/>
       </c>
     </row>
+    <row r="1531"/>
+    <row r="1532"/>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
@@ -16975,6 +17053,7 @@
         <v/>
       </c>
     </row>
+    <row r="1552"/>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
@@ -17028,6 +17107,8 @@
         <v/>
       </c>
     </row>
+    <row r="1557"/>
+    <row r="1558"/>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
@@ -17317,6 +17398,7 @@
         <v/>
       </c>
     </row>
+    <row r="1586"/>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
@@ -17370,6 +17452,7 @@
         <v/>
       </c>
     </row>
+    <row r="1591"/>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
@@ -17423,6 +17506,8 @@
         <v/>
       </c>
     </row>
+    <row r="1596"/>
+    <row r="1597"/>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
@@ -17586,6 +17671,7 @@
         <v/>
       </c>
     </row>
+    <row r="1613"/>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
@@ -17639,6 +17725,8 @@
         <v/>
       </c>
     </row>
+    <row r="1618"/>
+    <row r="1619"/>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
@@ -17907,6 +17995,7 @@
         <v/>
       </c>
     </row>
+    <row r="1645"/>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
@@ -17960,6 +18049,8 @@
         <v/>
       </c>
     </row>
+    <row r="1650"/>
+    <row r="1651"/>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
@@ -18186,6 +18277,7 @@
         <v/>
       </c>
     </row>
+    <row r="1673"/>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
@@ -18239,6 +18331,8 @@
         <v/>
       </c>
     </row>
+    <row r="1678"/>
+    <row r="1679"/>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
@@ -18402,6 +18496,7 @@
         <v/>
       </c>
     </row>
+    <row r="1695"/>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
@@ -18455,6 +18550,8 @@
         <v/>
       </c>
     </row>
+    <row r="1700"/>
+    <row r="1701"/>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
@@ -18681,6 +18778,7 @@
         <v/>
       </c>
     </row>
+    <row r="1723"/>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
@@ -18734,6 +18832,8 @@
         <v/>
       </c>
     </row>
+    <row r="1728"/>
+    <row r="1729"/>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
@@ -19191,6 +19291,7 @@
         <v/>
       </c>
     </row>
+    <row r="1773"/>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
@@ -19244,6 +19345,8 @@
         <v/>
       </c>
     </row>
+    <row r="1778"/>
+    <row r="1779"/>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
@@ -19449,6 +19552,7 @@
         <v/>
       </c>
     </row>
+    <row r="1799"/>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
@@ -19502,6 +19606,8 @@
         <v/>
       </c>
     </row>
+    <row r="1804"/>
+    <row r="1805"/>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
@@ -19770,6 +19876,7 @@
         <v/>
       </c>
     </row>
+    <row r="1831"/>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
@@ -19823,6 +19930,8 @@
         <v/>
       </c>
     </row>
+    <row r="1836"/>
+    <row r="1837"/>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
@@ -20049,6 +20158,7 @@
         <v/>
       </c>
     </row>
+    <row r="1859"/>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
@@ -20102,6 +20212,8 @@
         <v/>
       </c>
     </row>
+    <row r="1864"/>
+    <row r="1865"/>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
@@ -20407,6 +20519,7 @@
         <v/>
       </c>
     </row>
+    <row r="1894"/>
     <row r="1895">
       <c r="A1895" t="inlineStr">
         <is>
@@ -20460,6 +20573,7 @@
         <v/>
       </c>
     </row>
+    <row r="1899"/>
     <row r="1900">
       <c r="A1900" t="inlineStr">
         <is>
@@ -20623,6 +20737,7 @@
         <v/>
       </c>
     </row>
+    <row r="1915"/>
     <row r="1916">
       <c r="A1916" t="inlineStr">
         <is>
@@ -21009,6 +21124,8 @@
       </c>
       <c r="D1947" s="40" t="n"/>
     </row>
+    <row r="1948"/>
+    <row r="1949"/>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
@@ -21151,6 +21268,7 @@
         <v/>
       </c>
     </row>
+    <row r="1963"/>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
@@ -21204,6 +21322,8 @@
         <v/>
       </c>
     </row>
+    <row r="1968"/>
+    <row r="1969"/>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
@@ -21388,6 +21508,7 @@
         <v/>
       </c>
     </row>
+    <row r="1987"/>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
@@ -21441,6 +21562,8 @@
         <v/>
       </c>
     </row>
+    <row r="1992"/>
+    <row r="1993"/>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
@@ -21922,6 +22045,7 @@
         <v/>
       </c>
     </row>
+    <row r="2039"/>
     <row r="2040">
       <c r="A2040" t="inlineStr">
         <is>
@@ -21975,6 +22099,7 @@
         <v/>
       </c>
     </row>
+    <row r="2044"/>
     <row r="2045">
       <c r="A2045" t="inlineStr">
         <is>
@@ -21997,6 +22122,8 @@
         <v>-75360.2</v>
       </c>
     </row>
+    <row r="2047"/>
+    <row r="2048"/>
     <row r="2049">
       <c r="A2049" t="inlineStr">
         <is>
@@ -22391,6 +22518,7 @@
         <v/>
       </c>
     </row>
+    <row r="2086"/>
     <row r="2087">
       <c r="A2087" t="inlineStr">
         <is>
@@ -22444,6 +22572,8 @@
         <v/>
       </c>
     </row>
+    <row r="2091"/>
+    <row r="2092"/>
     <row r="2093">
       <c r="A2093" t="inlineStr">
         <is>
@@ -22565,6 +22695,7 @@
         <v/>
       </c>
     </row>
+    <row r="2104"/>
     <row r="2105">
       <c r="A2105" t="inlineStr">
         <is>
@@ -22618,6 +22749,8 @@
         <v/>
       </c>
     </row>
+    <row r="2109"/>
+    <row r="2110"/>
     <row r="2111">
       <c r="A2111" t="inlineStr">
         <is>
@@ -22886,6 +23019,7 @@
         <v/>
       </c>
     </row>
+    <row r="2136"/>
     <row r="2137">
       <c r="A2137" t="inlineStr">
         <is>
@@ -22939,6 +23073,8 @@
         <v/>
       </c>
     </row>
+    <row r="2141"/>
+    <row r="2142"/>
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
@@ -23186,6 +23322,7 @@
         <v/>
       </c>
     </row>
+    <row r="2166"/>
     <row r="2167">
       <c r="A2167" t="inlineStr">
         <is>
@@ -23239,6 +23376,8 @@
         <v/>
       </c>
     </row>
+    <row r="2171"/>
+    <row r="2172"/>
     <row r="2173">
       <c r="A2173" t="inlineStr">
         <is>
@@ -23444,6 +23583,7 @@
         <v/>
       </c>
     </row>
+    <row r="2192"/>
     <row r="2193">
       <c r="A2193" t="inlineStr">
         <is>
@@ -23497,6 +23637,8 @@
         <v/>
       </c>
     </row>
+    <row r="2197"/>
+    <row r="2198"/>
     <row r="2199">
       <c r="A2199" t="inlineStr">
         <is>
@@ -23681,6 +23823,7 @@
         <v/>
       </c>
     </row>
+    <row r="2216"/>
     <row r="2217">
       <c r="A2217" t="inlineStr">
         <is>
@@ -23734,6 +23877,8 @@
         <v/>
       </c>
     </row>
+    <row r="2221"/>
+    <row r="2222"/>
     <row r="2223">
       <c r="A2223" t="inlineStr">
         <is>
@@ -23876,6 +24021,7 @@
         <v/>
       </c>
     </row>
+    <row r="2236"/>
     <row r="2237">
       <c r="A2237" t="inlineStr">
         <is>
@@ -23929,6 +24075,8 @@
         <v/>
       </c>
     </row>
+    <row r="2241"/>
+    <row r="2242"/>
     <row r="2243">
       <c r="A2243" t="inlineStr">
         <is>
@@ -24197,6 +24345,7 @@
         <v/>
       </c>
     </row>
+    <row r="2268"/>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
@@ -24250,6 +24399,8 @@
         <v/>
       </c>
     </row>
+    <row r="2273"/>
+    <row r="2274"/>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
@@ -24560,6 +24711,7 @@
         <v/>
       </c>
     </row>
+    <row r="2304"/>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
@@ -24613,6 +24765,8 @@
         <v/>
       </c>
     </row>
+    <row r="2309"/>
+    <row r="2310"/>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
@@ -24797,6 +24951,7 @@
         <v/>
       </c>
     </row>
+    <row r="2328"/>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
@@ -24850,6 +25005,8 @@
         <v/>
       </c>
     </row>
+    <row r="2333"/>
+    <row r="2334"/>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
@@ -25076,6 +25233,7 @@
         <v/>
       </c>
     </row>
+    <row r="2356"/>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
@@ -25129,6 +25287,7 @@
         <v/>
       </c>
     </row>
+    <row r="2361"/>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
@@ -25152,6 +25311,8 @@
         <v/>
       </c>
     </row>
+    <row r="2364"/>
+    <row r="2365"/>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
@@ -25198,6 +25359,7 @@
         <v/>
       </c>
     </row>
+    <row r="2370"/>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
@@ -25250,6 +25412,8 @@
         <v/>
       </c>
     </row>
+    <row r="2375"/>
+    <row r="2376"/>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
@@ -25413,6 +25577,7 @@
         <v/>
       </c>
     </row>
+    <row r="2392"/>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
@@ -25466,6 +25631,8 @@
         <v/>
       </c>
     </row>
+    <row r="2397"/>
+    <row r="2398"/>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
@@ -25755,6 +25922,7 @@
         <v/>
       </c>
     </row>
+    <row r="2426"/>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
@@ -25808,6 +25976,8 @@
         <v/>
       </c>
     </row>
+    <row r="2431"/>
+    <row r="2432"/>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
@@ -26202,6 +26372,7 @@
         <v/>
       </c>
     </row>
+    <row r="2470"/>
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
@@ -26255,6 +26426,8 @@
         <v/>
       </c>
     </row>
+    <row r="2475"/>
+    <row r="2476"/>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
@@ -26481,6 +26654,7 @@
         <v/>
       </c>
     </row>
+    <row r="2498"/>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
@@ -26534,6 +26708,8 @@
         <v/>
       </c>
     </row>
+    <row r="2503"/>
+    <row r="2504"/>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
@@ -26844,6 +27020,7 @@
         <v/>
       </c>
     </row>
+    <row r="2534"/>
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
@@ -26897,6 +27074,8 @@
         <v/>
       </c>
     </row>
+    <row r="2539"/>
+    <row r="2540"/>
     <row r="2541">
       <c r="A2541" t="inlineStr">
         <is>
@@ -26943,6 +27122,7 @@
         <v/>
       </c>
     </row>
+    <row r="2545"/>
     <row r="2546">
       <c r="A2546" t="inlineStr">
         <is>
@@ -26965,6 +27145,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2548"/>
+    <row r="2549"/>
     <row r="2550">
       <c r="A2550" t="inlineStr">
         <is>
@@ -27011,6 +27193,7 @@
         <v/>
       </c>
     </row>
+    <row r="2554"/>
     <row r="2555">
       <c r="A2555" t="inlineStr">
         <is>
@@ -27033,6 +27216,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2557"/>
+    <row r="2558"/>
     <row r="2559">
       <c r="A2559" t="inlineStr">
         <is>
@@ -27091,6 +27276,7 @@
         <v/>
       </c>
     </row>
+    <row r="2564"/>
     <row r="2565">
       <c r="A2565" t="inlineStr">
         <is>
@@ -27144,6 +27330,7 @@
         <v/>
       </c>
     </row>
+    <row r="2569"/>
     <row r="2570">
       <c r="A2570" t="inlineStr">
         <is>
@@ -27166,7 +27353,9 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2574">
+    <row r="2572"/>
+    <row r="2573"/>
+    <row r="2574" s="44">
       <c r="A2574" t="inlineStr">
         <is>
           <t>2026.09.21</t>
@@ -27181,7 +27370,7 @@
         </is>
       </c>
     </row>
-    <row r="2575">
+    <row r="2575" s="44">
       <c r="A2575" t="n">
         <v>76905.41</v>
       </c>
@@ -27190,7 +27379,7 @@
         <v/>
       </c>
     </row>
-    <row r="2576">
+    <row r="2576" s="44">
       <c r="B2576" t="inlineStr">
         <is>
           <t xml:space="preserve">合計 </t>
@@ -27201,7 +27390,7 @@
         <v/>
       </c>
     </row>
-    <row r="2577">
+    <row r="2577" s="44">
       <c r="B2577" t="inlineStr">
         <is>
           <t>核驗</t>
@@ -27212,14 +27401,15 @@
         <v/>
       </c>
     </row>
-    <row r="2579">
+    <row r="2578" s="44"/>
+    <row r="2579" s="44">
       <c r="A2579" t="inlineStr">
         <is>
           <t>累積留倉   0股</t>
         </is>
       </c>
     </row>
-    <row r="2580">
+    <row r="2580" s="44">
       <c r="A2580" t="inlineStr">
         <is>
           <t>2026.09.10 留倉</t>
@@ -27248,7 +27438,7 @@
         <v/>
       </c>
     </row>
-    <row r="2582">
+    <row r="2582" s="44">
       <c r="A2582" s="41" t="inlineStr">
         <is>
           <t>2026.09.21 平倉</t>
@@ -27264,7 +27454,7 @@
         <v/>
       </c>
     </row>
-    <row r="2583">
+    <row r="2583" s="44">
       <c r="A2583" s="41" t="n"/>
       <c r="B2583" t="inlineStr">
         <is>
@@ -27276,7 +27466,7 @@
         <v/>
       </c>
     </row>
-    <row r="2584">
+    <row r="2584" s="44">
       <c r="A2584" s="41" t="n"/>
       <c r="B2584" t="inlineStr">
         <is>
@@ -27288,6 +27478,8 @@
         <v/>
       </c>
     </row>
+    <row r="2585"/>
+    <row r="2586"/>
     <row r="2587">
       <c r="A2587" t="inlineStr">
         <is>
@@ -27334,6 +27526,7 @@
         <v/>
       </c>
     </row>
+    <row r="2591"/>
     <row r="2592">
       <c r="A2592" t="inlineStr">
         <is>
@@ -27354,6 +27547,117 @@
       </c>
       <c r="C2593" t="n">
         <v>-76610.5</v>
+      </c>
+    </row>
+    <row r="2594"/>
+    <row r="2595"/>
+    <row r="2596">
+      <c r="A2596" t="inlineStr">
+        <is>
+          <t>2026.09.29</t>
+        </is>
+      </c>
+      <c r="B2596" s="81" t="n">
+        <v>40479.13</v>
+      </c>
+      <c r="C2596" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2597">
+      <c r="A2597" t="n">
+        <v>76353.5</v>
+      </c>
+      <c r="B2597">
+        <f>+B2596+A2597</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2598">
+      <c r="B2598" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2598">
+        <f>SUM(C2597:C2597)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2599">
+      <c r="B2599" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2599">
+        <f>+B2597-B2596-A2597</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2600"/>
+    <row r="2601">
+      <c r="A2601" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2602">
+      <c r="A2602" t="inlineStr">
+        <is>
+          <t>2026.09.28 留倉</t>
+        </is>
+      </c>
+      <c r="B2602" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2602" s="80" t="n">
+        <v>-76610.5</v>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" s="41" t="inlineStr">
+        <is>
+          <t>2026.09.29 平倉</t>
+        </is>
+      </c>
+      <c r="B2603" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2603" s="71">
+        <f>+A2597</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" s="41" t="n"/>
+      <c r="B2604" t="inlineStr">
+        <is>
+          <t>平倉損益</t>
+        </is>
+      </c>
+      <c r="C2604" s="80">
+        <f>+C2602+C2603</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" s="41" t="n"/>
+      <c r="B2605" t="inlineStr">
+        <is>
+          <t>平倉損益 %</t>
+        </is>
+      </c>
+      <c r="C2605" s="42">
+        <f>C2604/ABS(C2602)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -27368,7 +27672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -28182,6 +28486,18 @@
         <v/>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="86" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-257</v>
+      </c>
+      <c r="C68">
+        <f>C67+B68</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-16: ownership finalize (boss=_inbox/verify_shots/BOSS_SKILL_current), 9.0b docs, 10/15 ledgers
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2605"/>
+  <dimension ref="A1:E2619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -27598,64 +27598,196 @@
       </c>
     </row>
     <row r="2600"/>
-    <row r="2601">
-      <c r="A2601" t="inlineStr">
-        <is>
-          <t>累積留倉   0股</t>
-        </is>
-      </c>
-    </row>
+    <row r="2601"/>
     <row r="2602">
       <c r="A2602" t="inlineStr">
         <is>
+          <t>2026.10.15</t>
+        </is>
+      </c>
+      <c r="B2602" t="n">
+        <v>2382534.74</v>
+      </c>
+      <c r="C2602" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" t="n">
+        <v>-76993.67</v>
+      </c>
+      <c r="B2603">
+        <f>+B2602+A2603</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" t="n">
+        <v>77062.91</v>
+      </c>
+      <c r="B2604">
+        <f>+B2603+A2604</f>
+        <v/>
+      </c>
+      <c r="C2604" t="n">
+        <v>69.23999999999999</v>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" t="n">
+        <v>-77020</v>
+      </c>
+      <c r="B2605">
+        <f>+B2604+A2605</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" t="n">
+        <v>76998.42</v>
+      </c>
+      <c r="B2606">
+        <f>+B2605+A2606</f>
+        <v/>
+      </c>
+      <c r="C2606" t="n">
+        <v>-21.58</v>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="B2607" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2607" s="80">
+        <f>SUM(C2603:C2606)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="B2608" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2608" s="80">
+        <f>+B2606-B2602</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2610">
+      <c r="A2610" t="inlineStr">
+        <is>
+          <t>2026.10.15當沖</t>
+        </is>
+      </c>
+      <c r="B2610" t="inlineStr">
+        <is>
+          <t>買</t>
+        </is>
+      </c>
+      <c r="C2610" s="80">
+        <f>SUMIF(A2603:A2606,"&lt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2611">
+      <c r="A2611">
+        <f>"SPY " &amp; COUNT(C2603:C2606) * 100 &amp; "股"</f>
+        <v/>
+      </c>
+      <c r="B2611" t="inlineStr">
+        <is>
+          <t>賣</t>
+        </is>
+      </c>
+      <c r="C2611" s="80">
+        <f>SUMIF(A2603:A2606,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2612">
+      <c r="B2612" t="inlineStr">
+        <is>
+          <t>當日損益</t>
+        </is>
+      </c>
+      <c r="C2612" s="80">
+        <f>+C2610+C2611</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2613">
+      <c r="B2613" t="inlineStr">
+        <is>
+          <t>當日損益 %</t>
+        </is>
+      </c>
+      <c r="C2613" s="45">
+        <f>C2612/ABS(C2610)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2614"/>
+    <row r="2615">
+      <c r="A2615" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2616">
+      <c r="A2616" t="inlineStr">
+        <is>
           <t>2026.09.28 留倉</t>
         </is>
       </c>
-      <c r="B2602" t="inlineStr">
+      <c r="B2616" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2602" s="80" t="n">
+      <c r="C2616" t="n">
         <v>-76610.5</v>
       </c>
     </row>
-    <row r="2603">
-      <c r="A2603" s="41" t="inlineStr">
+    <row r="2617">
+      <c r="A2617" t="inlineStr">
         <is>
           <t>2026.09.29 平倉</t>
         </is>
       </c>
-      <c r="B2603" t="inlineStr">
+      <c r="B2617" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2603" s="71">
+      <c r="C2617">
         <f>+A2597</f>
         <v/>
       </c>
     </row>
-    <row r="2604">
-      <c r="A2604" s="41" t="n"/>
-      <c r="B2604" t="inlineStr">
+    <row r="2618">
+      <c r="B2618" t="inlineStr">
         <is>
           <t>平倉損益</t>
         </is>
       </c>
-      <c r="C2604" s="80">
+      <c r="C2618">
         <f>+C2602+C2603</f>
         <v/>
       </c>
     </row>
-    <row r="2605">
-      <c r="A2605" s="41" t="n"/>
-      <c r="B2605" t="inlineStr">
+    <row r="2619">
+      <c r="B2619" t="inlineStr">
         <is>
           <t>平倉損益 %</t>
         </is>
       </c>
-      <c r="C2605" s="42">
+      <c r="C2619">
         <f>C2604/ABS(C2602)</f>
         <v/>
       </c>
@@ -27672,7 +27804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -28498,6 +28630,18 @@
         <v/>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="86" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B69" t="n">
+        <v>47.66</v>
+      </c>
+      <c r="C69">
+        <f>C68+B69</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-19: 10/16 manual commit (daytrade+overnight 300sh), fix C2618/C2619 refs, offset note
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2619"/>
+  <dimension ref="A1:D2639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -11266,8 +11266,6 @@
         <v/>
       </c>
     </row>
-    <row r="975"/>
-    <row r="976"/>
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
@@ -11464,7 +11462,6 @@
         <v/>
       </c>
     </row>
-    <row r="996"/>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
@@ -11518,8 +11515,6 @@
         <v/>
       </c>
     </row>
-    <row r="1001"/>
-    <row r="1002"/>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
@@ -11559,8 +11554,6 @@
         <v/>
       </c>
     </row>
-    <row r="1006"/>
-    <row r="1007"/>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
@@ -11682,7 +11675,6 @@
         <v/>
       </c>
     </row>
-    <row r="1019"/>
     <row r="1020">
       <c r="A1020" t="inlineStr">
         <is>
@@ -11736,8 +11728,6 @@
         <v/>
       </c>
     </row>
-    <row r="1024"/>
-    <row r="1025"/>
     <row r="1026">
       <c r="A1026" t="inlineStr">
         <is>
@@ -11777,8 +11767,6 @@
         <v/>
       </c>
     </row>
-    <row r="1029"/>
-    <row r="1030"/>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
@@ -11840,7 +11828,6 @@
         <v/>
       </c>
     </row>
-    <row r="1036"/>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
@@ -11848,7 +11835,6 @@
         </is>
       </c>
     </row>
-    <row r="1038"/>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
@@ -11903,7 +11889,6 @@
         <v/>
       </c>
     </row>
-    <row r="1043"/>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
@@ -11958,7 +11943,6 @@
         <v/>
       </c>
     </row>
-    <row r="1048"/>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
@@ -12080,7 +12064,6 @@
         <v/>
       </c>
     </row>
-    <row r="1060"/>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
@@ -12134,8 +12117,6 @@
         <v/>
       </c>
     </row>
-    <row r="1065"/>
-    <row r="1066"/>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
@@ -12266,7 +12247,6 @@
         <v/>
       </c>
     </row>
-    <row r="1079"/>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
@@ -12320,7 +12300,6 @@
         <v/>
       </c>
     </row>
-    <row r="1084"/>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
@@ -12343,8 +12322,6 @@
         <v>-75037.94</v>
       </c>
     </row>
-    <row r="1087"/>
-    <row r="1088"/>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
@@ -12496,7 +12473,6 @@
         <v/>
       </c>
     </row>
-    <row r="1103"/>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
@@ -12550,7 +12526,6 @@
         <v/>
       </c>
     </row>
-    <row r="1108"/>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
@@ -12604,8 +12579,6 @@
         <v/>
       </c>
     </row>
-    <row r="1113"/>
-    <row r="1114"/>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
@@ -12706,7 +12679,6 @@
         <v/>
       </c>
     </row>
-    <row r="1124"/>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
@@ -12760,8 +12732,6 @@
         <v/>
       </c>
     </row>
-    <row r="1129"/>
-    <row r="1130"/>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
@@ -12925,7 +12895,6 @@
         <v/>
       </c>
     </row>
-    <row r="1146"/>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
@@ -12979,8 +12948,6 @@
         <v/>
       </c>
     </row>
-    <row r="1151"/>
-    <row r="1152"/>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
@@ -13144,7 +13111,6 @@
         <v/>
       </c>
     </row>
-    <row r="1168"/>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
@@ -13198,8 +13164,6 @@
         <v/>
       </c>
     </row>
-    <row r="1173"/>
-    <row r="1174"/>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
@@ -13369,7 +13333,6 @@
         <v/>
       </c>
     </row>
-    <row r="1191"/>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
@@ -13423,7 +13386,6 @@
         <v/>
       </c>
     </row>
-    <row r="1196"/>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
@@ -13476,8 +13438,6 @@
         <v>-74653</v>
       </c>
     </row>
-    <row r="1201"/>
-    <row r="1202"/>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
@@ -13608,7 +13568,6 @@
         <v/>
       </c>
     </row>
-    <row r="1215"/>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
@@ -13662,7 +13621,6 @@
         <v/>
       </c>
     </row>
-    <row r="1220"/>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
@@ -13716,7 +13674,6 @@
         <v/>
       </c>
     </row>
-    <row r="1225"/>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
@@ -13756,8 +13713,6 @@
         <v/>
       </c>
     </row>
-    <row r="1229"/>
-    <row r="1230"/>
     <row r="1231">
       <c r="A1231" s="80" t="inlineStr">
         <is>
@@ -14089,7 +14044,6 @@
         <v/>
       </c>
     </row>
-    <row r="1261"/>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
@@ -14143,7 +14097,6 @@
         <v/>
       </c>
     </row>
-    <row r="1266"/>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
@@ -14198,8 +14151,6 @@
         <v>-74291.5</v>
       </c>
     </row>
-    <row r="1271"/>
-    <row r="1272"/>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
@@ -14531,7 +14482,6 @@
         <v/>
       </c>
     </row>
-    <row r="1305"/>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
@@ -14585,7 +14535,6 @@
         <v/>
       </c>
     </row>
-    <row r="1310"/>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
@@ -14641,8 +14590,6 @@
         <v/>
       </c>
     </row>
-    <row r="1315"/>
-    <row r="1316"/>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
@@ -14878,7 +14825,6 @@
         <v/>
       </c>
     </row>
-    <row r="1339"/>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
@@ -14932,7 +14878,6 @@
         <v/>
       </c>
     </row>
-    <row r="1344"/>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
@@ -15003,7 +14948,6 @@
         <v>-72794.59</v>
       </c>
     </row>
-    <row r="1350"/>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
@@ -15188,7 +15132,6 @@
         <v/>
       </c>
     </row>
-    <row r="1368"/>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
@@ -15242,7 +15185,6 @@
         <v/>
       </c>
     </row>
-    <row r="1373"/>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
@@ -15314,7 +15256,6 @@
         <v/>
       </c>
     </row>
-    <row r="1379"/>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
@@ -15430,7 +15371,6 @@
         <v/>
       </c>
     </row>
-    <row r="1391"/>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
@@ -15484,7 +15424,6 @@
         <v/>
       </c>
     </row>
-    <row r="1396"/>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
@@ -15534,7 +15473,6 @@
         <v/>
       </c>
     </row>
-    <row r="1401"/>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
@@ -15584,7 +15522,6 @@
         <v/>
       </c>
     </row>
-    <row r="1406"/>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
@@ -15634,7 +15571,6 @@
         <v/>
       </c>
     </row>
-    <row r="1411"/>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
@@ -15684,8 +15620,6 @@
         <v/>
       </c>
     </row>
-    <row r="1416"/>
-    <row r="1417"/>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
@@ -15858,7 +15792,6 @@
         <v/>
       </c>
     </row>
-    <row r="1434"/>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
@@ -15915,7 +15848,6 @@
         <v/>
       </c>
     </row>
-    <row r="1439"/>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
@@ -15938,7 +15870,6 @@
         <v>-75313</v>
       </c>
     </row>
-    <row r="1442"/>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
@@ -16291,7 +16222,6 @@
         <v/>
       </c>
     </row>
-    <row r="1476"/>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
@@ -16345,8 +16275,6 @@
         <v/>
       </c>
     </row>
-    <row r="1481"/>
-    <row r="1482"/>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
@@ -16552,7 +16480,6 @@
         <v/>
       </c>
     </row>
-    <row r="1502"/>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
@@ -16606,8 +16533,6 @@
         <v/>
       </c>
     </row>
-    <row r="1507"/>
-    <row r="1508"/>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
@@ -16792,7 +16717,6 @@
         <v/>
       </c>
     </row>
-    <row r="1526"/>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
@@ -16846,8 +16770,6 @@
         <v/>
       </c>
     </row>
-    <row r="1531"/>
-    <row r="1532"/>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
@@ -17053,7 +16975,6 @@
         <v/>
       </c>
     </row>
-    <row r="1552"/>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
@@ -17107,8 +17028,6 @@
         <v/>
       </c>
     </row>
-    <row r="1557"/>
-    <row r="1558"/>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
@@ -17398,7 +17317,6 @@
         <v/>
       </c>
     </row>
-    <row r="1586"/>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
@@ -17452,7 +17370,6 @@
         <v/>
       </c>
     </row>
-    <row r="1591"/>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
@@ -17506,8 +17423,6 @@
         <v/>
       </c>
     </row>
-    <row r="1596"/>
-    <row r="1597"/>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
@@ -17671,7 +17586,6 @@
         <v/>
       </c>
     </row>
-    <row r="1613"/>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
@@ -17725,8 +17639,6 @@
         <v/>
       </c>
     </row>
-    <row r="1618"/>
-    <row r="1619"/>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
@@ -17995,7 +17907,6 @@
         <v/>
       </c>
     </row>
-    <row r="1645"/>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
@@ -18049,8 +17960,6 @@
         <v/>
       </c>
     </row>
-    <row r="1650"/>
-    <row r="1651"/>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
@@ -18277,7 +18186,6 @@
         <v/>
       </c>
     </row>
-    <row r="1673"/>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
@@ -18331,8 +18239,6 @@
         <v/>
       </c>
     </row>
-    <row r="1678"/>
-    <row r="1679"/>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
@@ -18496,7 +18402,6 @@
         <v/>
       </c>
     </row>
-    <row r="1695"/>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
@@ -18550,8 +18455,6 @@
         <v/>
       </c>
     </row>
-    <row r="1700"/>
-    <row r="1701"/>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
@@ -18778,7 +18681,6 @@
         <v/>
       </c>
     </row>
-    <row r="1723"/>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
@@ -18832,8 +18734,6 @@
         <v/>
       </c>
     </row>
-    <row r="1728"/>
-    <row r="1729"/>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
@@ -19291,7 +19191,6 @@
         <v/>
       </c>
     </row>
-    <row r="1773"/>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
@@ -19345,8 +19244,6 @@
         <v/>
       </c>
     </row>
-    <row r="1778"/>
-    <row r="1779"/>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
@@ -19552,7 +19449,6 @@
         <v/>
       </c>
     </row>
-    <row r="1799"/>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
@@ -19606,8 +19502,6 @@
         <v/>
       </c>
     </row>
-    <row r="1804"/>
-    <row r="1805"/>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
@@ -19876,7 +19770,6 @@
         <v/>
       </c>
     </row>
-    <row r="1831"/>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
@@ -19930,8 +19823,6 @@
         <v/>
       </c>
     </row>
-    <row r="1836"/>
-    <row r="1837"/>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
@@ -20158,7 +20049,6 @@
         <v/>
       </c>
     </row>
-    <row r="1859"/>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
@@ -20212,8 +20102,6 @@
         <v/>
       </c>
     </row>
-    <row r="1864"/>
-    <row r="1865"/>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
@@ -20519,7 +20407,6 @@
         <v/>
       </c>
     </row>
-    <row r="1894"/>
     <row r="1895">
       <c r="A1895" t="inlineStr">
         <is>
@@ -20573,7 +20460,6 @@
         <v/>
       </c>
     </row>
-    <row r="1899"/>
     <row r="1900">
       <c r="A1900" t="inlineStr">
         <is>
@@ -20737,7 +20623,6 @@
         <v/>
       </c>
     </row>
-    <row r="1915"/>
     <row r="1916">
       <c r="A1916" t="inlineStr">
         <is>
@@ -21124,8 +21009,6 @@
       </c>
       <c r="D1947" s="40" t="n"/>
     </row>
-    <row r="1948"/>
-    <row r="1949"/>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
@@ -21268,7 +21151,6 @@
         <v/>
       </c>
     </row>
-    <row r="1963"/>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
@@ -21322,8 +21204,6 @@
         <v/>
       </c>
     </row>
-    <row r="1968"/>
-    <row r="1969"/>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
@@ -21508,7 +21388,6 @@
         <v/>
       </c>
     </row>
-    <row r="1987"/>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
@@ -21562,8 +21441,6 @@
         <v/>
       </c>
     </row>
-    <row r="1992"/>
-    <row r="1993"/>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
@@ -22045,7 +21922,6 @@
         <v/>
       </c>
     </row>
-    <row r="2039"/>
     <row r="2040">
       <c r="A2040" t="inlineStr">
         <is>
@@ -22099,7 +21975,6 @@
         <v/>
       </c>
     </row>
-    <row r="2044"/>
     <row r="2045">
       <c r="A2045" t="inlineStr">
         <is>
@@ -22122,8 +21997,6 @@
         <v>-75360.2</v>
       </c>
     </row>
-    <row r="2047"/>
-    <row r="2048"/>
     <row r="2049">
       <c r="A2049" t="inlineStr">
         <is>
@@ -22518,7 +22391,6 @@
         <v/>
       </c>
     </row>
-    <row r="2086"/>
     <row r="2087">
       <c r="A2087" t="inlineStr">
         <is>
@@ -22572,8 +22444,6 @@
         <v/>
       </c>
     </row>
-    <row r="2091"/>
-    <row r="2092"/>
     <row r="2093">
       <c r="A2093" t="inlineStr">
         <is>
@@ -22695,7 +22565,6 @@
         <v/>
       </c>
     </row>
-    <row r="2104"/>
     <row r="2105">
       <c r="A2105" t="inlineStr">
         <is>
@@ -22749,8 +22618,6 @@
         <v/>
       </c>
     </row>
-    <row r="2109"/>
-    <row r="2110"/>
     <row r="2111">
       <c r="A2111" t="inlineStr">
         <is>
@@ -23019,7 +22886,6 @@
         <v/>
       </c>
     </row>
-    <row r="2136"/>
     <row r="2137">
       <c r="A2137" t="inlineStr">
         <is>
@@ -23073,8 +22939,6 @@
         <v/>
       </c>
     </row>
-    <row r="2141"/>
-    <row r="2142"/>
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
@@ -23322,7 +23186,6 @@
         <v/>
       </c>
     </row>
-    <row r="2166"/>
     <row r="2167">
       <c r="A2167" t="inlineStr">
         <is>
@@ -23376,8 +23239,6 @@
         <v/>
       </c>
     </row>
-    <row r="2171"/>
-    <row r="2172"/>
     <row r="2173">
       <c r="A2173" t="inlineStr">
         <is>
@@ -23583,7 +23444,6 @@
         <v/>
       </c>
     </row>
-    <row r="2192"/>
     <row r="2193">
       <c r="A2193" t="inlineStr">
         <is>
@@ -23637,8 +23497,6 @@
         <v/>
       </c>
     </row>
-    <row r="2197"/>
-    <row r="2198"/>
     <row r="2199">
       <c r="A2199" t="inlineStr">
         <is>
@@ -23823,7 +23681,6 @@
         <v/>
       </c>
     </row>
-    <row r="2216"/>
     <row r="2217">
       <c r="A2217" t="inlineStr">
         <is>
@@ -23877,8 +23734,6 @@
         <v/>
       </c>
     </row>
-    <row r="2221"/>
-    <row r="2222"/>
     <row r="2223">
       <c r="A2223" t="inlineStr">
         <is>
@@ -24021,7 +23876,6 @@
         <v/>
       </c>
     </row>
-    <row r="2236"/>
     <row r="2237">
       <c r="A2237" t="inlineStr">
         <is>
@@ -24075,8 +23929,6 @@
         <v/>
       </c>
     </row>
-    <row r="2241"/>
-    <row r="2242"/>
     <row r="2243">
       <c r="A2243" t="inlineStr">
         <is>
@@ -24345,7 +24197,6 @@
         <v/>
       </c>
     </row>
-    <row r="2268"/>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
@@ -24399,8 +24250,6 @@
         <v/>
       </c>
     </row>
-    <row r="2273"/>
-    <row r="2274"/>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
@@ -24711,7 +24560,6 @@
         <v/>
       </c>
     </row>
-    <row r="2304"/>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
@@ -24765,8 +24613,6 @@
         <v/>
       </c>
     </row>
-    <row r="2309"/>
-    <row r="2310"/>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
@@ -24951,7 +24797,6 @@
         <v/>
       </c>
     </row>
-    <row r="2328"/>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
@@ -25005,8 +24850,6 @@
         <v/>
       </c>
     </row>
-    <row r="2333"/>
-    <row r="2334"/>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
@@ -25233,7 +25076,6 @@
         <v/>
       </c>
     </row>
-    <row r="2356"/>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
@@ -25287,7 +25129,6 @@
         <v/>
       </c>
     </row>
-    <row r="2361"/>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
@@ -25311,8 +25152,6 @@
         <v/>
       </c>
     </row>
-    <row r="2364"/>
-    <row r="2365"/>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
@@ -25359,7 +25198,6 @@
         <v/>
       </c>
     </row>
-    <row r="2370"/>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
@@ -25412,8 +25250,6 @@
         <v/>
       </c>
     </row>
-    <row r="2375"/>
-    <row r="2376"/>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
@@ -25577,7 +25413,6 @@
         <v/>
       </c>
     </row>
-    <row r="2392"/>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
@@ -25631,8 +25466,6 @@
         <v/>
       </c>
     </row>
-    <row r="2397"/>
-    <row r="2398"/>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
@@ -25922,7 +25755,6 @@
         <v/>
       </c>
     </row>
-    <row r="2426"/>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
@@ -25976,8 +25808,6 @@
         <v/>
       </c>
     </row>
-    <row r="2431"/>
-    <row r="2432"/>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
@@ -26372,7 +26202,6 @@
         <v/>
       </c>
     </row>
-    <row r="2470"/>
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
@@ -26426,8 +26255,6 @@
         <v/>
       </c>
     </row>
-    <row r="2475"/>
-    <row r="2476"/>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
@@ -26654,7 +26481,6 @@
         <v/>
       </c>
     </row>
-    <row r="2498"/>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
@@ -26708,8 +26534,6 @@
         <v/>
       </c>
     </row>
-    <row r="2503"/>
-    <row r="2504"/>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
@@ -27020,7 +26844,6 @@
         <v/>
       </c>
     </row>
-    <row r="2534"/>
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
@@ -27074,8 +26897,6 @@
         <v/>
       </c>
     </row>
-    <row r="2539"/>
-    <row r="2540"/>
     <row r="2541">
       <c r="A2541" t="inlineStr">
         <is>
@@ -27122,7 +26943,6 @@
         <v/>
       </c>
     </row>
-    <row r="2545"/>
     <row r="2546">
       <c r="A2546" t="inlineStr">
         <is>
@@ -27145,8 +26965,6 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2548"/>
-    <row r="2549"/>
     <row r="2550">
       <c r="A2550" t="inlineStr">
         <is>
@@ -27193,7 +27011,6 @@
         <v/>
       </c>
     </row>
-    <row r="2554"/>
     <row r="2555">
       <c r="A2555" t="inlineStr">
         <is>
@@ -27216,8 +27033,6 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2557"/>
-    <row r="2558"/>
     <row r="2559">
       <c r="A2559" t="inlineStr">
         <is>
@@ -27276,7 +27091,6 @@
         <v/>
       </c>
     </row>
-    <row r="2564"/>
     <row r="2565">
       <c r="A2565" t="inlineStr">
         <is>
@@ -27330,7 +27144,6 @@
         <v/>
       </c>
     </row>
-    <row r="2569"/>
     <row r="2570">
       <c r="A2570" t="inlineStr">
         <is>
@@ -27353,8 +27166,6 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2572"/>
-    <row r="2573"/>
     <row r="2574" s="44">
       <c r="A2574" t="inlineStr">
         <is>
@@ -27478,8 +27289,6 @@
         <v/>
       </c>
     </row>
-    <row r="2585"/>
-    <row r="2586"/>
     <row r="2587">
       <c r="A2587" t="inlineStr">
         <is>
@@ -27526,7 +27335,6 @@
         <v/>
       </c>
     </row>
-    <row r="2591"/>
     <row r="2592">
       <c r="A2592" t="inlineStr">
         <is>
@@ -27549,8 +27357,6 @@
         <v>-76610.5</v>
       </c>
     </row>
-    <row r="2594"/>
-    <row r="2595"/>
     <row r="2596">
       <c r="A2596" t="inlineStr">
         <is>
@@ -27597,8 +27403,6 @@
         <v/>
       </c>
     </row>
-    <row r="2600"/>
-    <row r="2601"/>
     <row r="2602">
       <c r="A2602" t="inlineStr">
         <is>
@@ -27731,7 +27535,6 @@
         <v/>
       </c>
     </row>
-    <row r="2614"/>
     <row r="2615">
       <c r="A2615" t="inlineStr">
         <is>
@@ -27777,7 +27580,7 @@
         </is>
       </c>
       <c r="C2618">
-        <f>+C2602+C2603</f>
+        <f>+C2616+C2617</f>
         <v/>
       </c>
     </row>
@@ -27788,8 +27591,198 @@
         </is>
       </c>
       <c r="C2619">
-        <f>C2604/ABS(C2602)</f>
-        <v/>
+        <f>C2618/ABS(C2616)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2622">
+      <c r="A2622" t="inlineStr">
+        <is>
+          <t>2026.10.16</t>
+        </is>
+      </c>
+      <c r="B2622" t="n">
+        <v>2382534.74</v>
+      </c>
+      <c r="C2622" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2623">
+      <c r="A2623" t="n">
+        <v>-76763.5</v>
+      </c>
+      <c r="B2623">
+        <f>+B2622+A2623</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2624">
+      <c r="A2624" t="n">
+        <v>76776.78999999999</v>
+      </c>
+      <c r="B2624">
+        <f>+B2623+A2624</f>
+        <v/>
+      </c>
+      <c r="C2624" t="n">
+        <v>13.29</v>
+      </c>
+    </row>
+    <row r="2625">
+      <c r="A2625" t="n">
+        <v>-76663.96000000001</v>
+      </c>
+      <c r="B2625">
+        <f>+B2624+A2625</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2626">
+      <c r="A2626" t="n">
+        <v>-76592.61</v>
+      </c>
+      <c r="B2626">
+        <f>+B2625+A2626</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2627">
+      <c r="A2627" t="n">
+        <v>-76401</v>
+      </c>
+      <c r="B2627">
+        <f>+B2626+A2627</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2628">
+      <c r="B2628" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2628" s="80">
+        <f>SUM(C2623:C2627)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2629">
+      <c r="B2629" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2629" s="80">
+        <f>+B2627-B2622-A2625-A2626-A2627</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2631">
+      <c r="A2631" t="inlineStr">
+        <is>
+          <t>2026.10.16當沖</t>
+        </is>
+      </c>
+      <c r="B2631" t="inlineStr">
+        <is>
+          <t>買</t>
+        </is>
+      </c>
+      <c r="C2631" s="80">
+        <f>SUMIF(A2623:A2624,"&lt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2632">
+      <c r="A2632">
+        <f>"SPY " &amp; COUNT(C2623:C2624) * 100 &amp; "股"</f>
+        <v/>
+      </c>
+      <c r="B2632" t="inlineStr">
+        <is>
+          <t>賣</t>
+        </is>
+      </c>
+      <c r="C2632" s="80">
+        <f>SUMIF(A2623:A2624,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2633">
+      <c r="B2633" t="inlineStr">
+        <is>
+          <t>當日損益</t>
+        </is>
+      </c>
+      <c r="C2633" s="80">
+        <f>+C2631+C2632</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2634">
+      <c r="B2634" t="inlineStr">
+        <is>
+          <t>當日損益 %</t>
+        </is>
+      </c>
+      <c r="C2634" s="45">
+        <f>C2633/ABS(C2631)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2636">
+      <c r="A2636" t="inlineStr">
+        <is>
+          <t>累積留倉   300股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2637">
+      <c r="A2637" t="inlineStr">
+        <is>
+          <t>2026.10.16 留倉</t>
+        </is>
+      </c>
+      <c r="B2637" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2637" t="n">
+        <v>-76663.96000000001</v>
+      </c>
+    </row>
+    <row r="2638">
+      <c r="A2638" t="inlineStr">
+        <is>
+          <t>2026.10.16 留倉</t>
+        </is>
+      </c>
+      <c r="B2638" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2638" t="n">
+        <v>-76592.61</v>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" t="inlineStr">
+        <is>
+          <t>2026.10.16 留倉</t>
+        </is>
+      </c>
+      <c r="B2639" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2639" t="n">
+        <v>-76401</v>
       </c>
     </row>
   </sheetData>
@@ -27804,7 +27797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -28642,6 +28635,18 @@
         <v/>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="86" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B70" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="C70">
+        <f>C69+B70</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-20 12:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2639"/>
+  <dimension ref="A1:D2652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -11266,6 +11266,8 @@
         <v/>
       </c>
     </row>
+    <row r="975"/>
+    <row r="976"/>
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
@@ -11462,6 +11464,7 @@
         <v/>
       </c>
     </row>
+    <row r="996"/>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
@@ -11515,6 +11518,8 @@
         <v/>
       </c>
     </row>
+    <row r="1001"/>
+    <row r="1002"/>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
@@ -11554,6 +11559,8 @@
         <v/>
       </c>
     </row>
+    <row r="1006"/>
+    <row r="1007"/>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
@@ -11675,6 +11682,7 @@
         <v/>
       </c>
     </row>
+    <row r="1019"/>
     <row r="1020">
       <c r="A1020" t="inlineStr">
         <is>
@@ -11728,6 +11736,8 @@
         <v/>
       </c>
     </row>
+    <row r="1024"/>
+    <row r="1025"/>
     <row r="1026">
       <c r="A1026" t="inlineStr">
         <is>
@@ -11767,6 +11777,8 @@
         <v/>
       </c>
     </row>
+    <row r="1029"/>
+    <row r="1030"/>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
@@ -11828,6 +11840,7 @@
         <v/>
       </c>
     </row>
+    <row r="1036"/>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
@@ -11835,6 +11848,7 @@
         </is>
       </c>
     </row>
+    <row r="1038"/>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
@@ -11889,6 +11903,7 @@
         <v/>
       </c>
     </row>
+    <row r="1043"/>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
@@ -11943,6 +11958,7 @@
         <v/>
       </c>
     </row>
+    <row r="1048"/>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
@@ -12064,6 +12080,7 @@
         <v/>
       </c>
     </row>
+    <row r="1060"/>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
@@ -12117,6 +12134,8 @@
         <v/>
       </c>
     </row>
+    <row r="1065"/>
+    <row r="1066"/>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
@@ -12247,6 +12266,7 @@
         <v/>
       </c>
     </row>
+    <row r="1079"/>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
@@ -12300,6 +12320,7 @@
         <v/>
       </c>
     </row>
+    <row r="1084"/>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
@@ -12322,6 +12343,8 @@
         <v>-75037.94</v>
       </c>
     </row>
+    <row r="1087"/>
+    <row r="1088"/>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
@@ -12473,6 +12496,7 @@
         <v/>
       </c>
     </row>
+    <row r="1103"/>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
@@ -12526,6 +12550,7 @@
         <v/>
       </c>
     </row>
+    <row r="1108"/>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
@@ -12579,6 +12604,8 @@
         <v/>
       </c>
     </row>
+    <row r="1113"/>
+    <row r="1114"/>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
@@ -12679,6 +12706,7 @@
         <v/>
       </c>
     </row>
+    <row r="1124"/>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
@@ -12732,6 +12760,8 @@
         <v/>
       </c>
     </row>
+    <row r="1129"/>
+    <row r="1130"/>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
@@ -12895,6 +12925,7 @@
         <v/>
       </c>
     </row>
+    <row r="1146"/>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
@@ -12948,6 +12979,8 @@
         <v/>
       </c>
     </row>
+    <row r="1151"/>
+    <row r="1152"/>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
@@ -13111,6 +13144,7 @@
         <v/>
       </c>
     </row>
+    <row r="1168"/>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
@@ -13164,6 +13198,8 @@
         <v/>
       </c>
     </row>
+    <row r="1173"/>
+    <row r="1174"/>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
@@ -13333,6 +13369,7 @@
         <v/>
       </c>
     </row>
+    <row r="1191"/>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
@@ -13386,6 +13423,7 @@
         <v/>
       </c>
     </row>
+    <row r="1196"/>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
@@ -13438,6 +13476,8 @@
         <v>-74653</v>
       </c>
     </row>
+    <row r="1201"/>
+    <row r="1202"/>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
@@ -13568,6 +13608,7 @@
         <v/>
       </c>
     </row>
+    <row r="1215"/>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
@@ -13621,6 +13662,7 @@
         <v/>
       </c>
     </row>
+    <row r="1220"/>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
@@ -13674,6 +13716,7 @@
         <v/>
       </c>
     </row>
+    <row r="1225"/>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
@@ -13713,6 +13756,8 @@
         <v/>
       </c>
     </row>
+    <row r="1229"/>
+    <row r="1230"/>
     <row r="1231">
       <c r="A1231" s="80" t="inlineStr">
         <is>
@@ -14044,6 +14089,7 @@
         <v/>
       </c>
     </row>
+    <row r="1261"/>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
@@ -14097,6 +14143,7 @@
         <v/>
       </c>
     </row>
+    <row r="1266"/>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
@@ -14151,6 +14198,8 @@
         <v>-74291.5</v>
       </c>
     </row>
+    <row r="1271"/>
+    <row r="1272"/>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
@@ -14482,6 +14531,7 @@
         <v/>
       </c>
     </row>
+    <row r="1305"/>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
@@ -14535,6 +14585,7 @@
         <v/>
       </c>
     </row>
+    <row r="1310"/>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
@@ -14590,6 +14641,8 @@
         <v/>
       </c>
     </row>
+    <row r="1315"/>
+    <row r="1316"/>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
@@ -14825,6 +14878,7 @@
         <v/>
       </c>
     </row>
+    <row r="1339"/>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
@@ -14878,6 +14932,7 @@
         <v/>
       </c>
     </row>
+    <row r="1344"/>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
@@ -14948,6 +15003,7 @@
         <v>-72794.59</v>
       </c>
     </row>
+    <row r="1350"/>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
@@ -15132,6 +15188,7 @@
         <v/>
       </c>
     </row>
+    <row r="1368"/>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
@@ -15185,6 +15242,7 @@
         <v/>
       </c>
     </row>
+    <row r="1373"/>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
@@ -15256,6 +15314,7 @@
         <v/>
       </c>
     </row>
+    <row r="1379"/>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
@@ -15371,6 +15430,7 @@
         <v/>
       </c>
     </row>
+    <row r="1391"/>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
@@ -15424,6 +15484,7 @@
         <v/>
       </c>
     </row>
+    <row r="1396"/>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
@@ -15473,6 +15534,7 @@
         <v/>
       </c>
     </row>
+    <row r="1401"/>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
@@ -15522,6 +15584,7 @@
         <v/>
       </c>
     </row>
+    <row r="1406"/>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
@@ -15571,6 +15634,7 @@
         <v/>
       </c>
     </row>
+    <row r="1411"/>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
@@ -15620,6 +15684,8 @@
         <v/>
       </c>
     </row>
+    <row r="1416"/>
+    <row r="1417"/>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
@@ -15792,6 +15858,7 @@
         <v/>
       </c>
     </row>
+    <row r="1434"/>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
@@ -15848,6 +15915,7 @@
         <v/>
       </c>
     </row>
+    <row r="1439"/>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
@@ -15870,6 +15938,7 @@
         <v>-75313</v>
       </c>
     </row>
+    <row r="1442"/>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
@@ -16222,6 +16291,7 @@
         <v/>
       </c>
     </row>
+    <row r="1476"/>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
@@ -16275,6 +16345,8 @@
         <v/>
       </c>
     </row>
+    <row r="1481"/>
+    <row r="1482"/>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
@@ -16480,6 +16552,7 @@
         <v/>
       </c>
     </row>
+    <row r="1502"/>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
@@ -16533,6 +16606,8 @@
         <v/>
       </c>
     </row>
+    <row r="1507"/>
+    <row r="1508"/>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
@@ -16717,6 +16792,7 @@
         <v/>
       </c>
     </row>
+    <row r="1526"/>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
@@ -16770,6 +16846,8 @@
         <v/>
       </c>
     </row>
+    <row r="1531"/>
+    <row r="1532"/>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
@@ -16975,6 +17053,7 @@
         <v/>
       </c>
     </row>
+    <row r="1552"/>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
@@ -17028,6 +17107,8 @@
         <v/>
       </c>
     </row>
+    <row r="1557"/>
+    <row r="1558"/>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
@@ -17317,6 +17398,7 @@
         <v/>
       </c>
     </row>
+    <row r="1586"/>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
@@ -17370,6 +17452,7 @@
         <v/>
       </c>
     </row>
+    <row r="1591"/>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
@@ -17423,6 +17506,8 @@
         <v/>
       </c>
     </row>
+    <row r="1596"/>
+    <row r="1597"/>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
@@ -17586,6 +17671,7 @@
         <v/>
       </c>
     </row>
+    <row r="1613"/>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
@@ -17639,6 +17725,8 @@
         <v/>
       </c>
     </row>
+    <row r="1618"/>
+    <row r="1619"/>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
@@ -17907,6 +17995,7 @@
         <v/>
       </c>
     </row>
+    <row r="1645"/>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
@@ -17960,6 +18049,8 @@
         <v/>
       </c>
     </row>
+    <row r="1650"/>
+    <row r="1651"/>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
@@ -18186,6 +18277,7 @@
         <v/>
       </c>
     </row>
+    <row r="1673"/>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
@@ -18239,6 +18331,8 @@
         <v/>
       </c>
     </row>
+    <row r="1678"/>
+    <row r="1679"/>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
@@ -18402,6 +18496,7 @@
         <v/>
       </c>
     </row>
+    <row r="1695"/>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
@@ -18455,6 +18550,8 @@
         <v/>
       </c>
     </row>
+    <row r="1700"/>
+    <row r="1701"/>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
@@ -18681,6 +18778,7 @@
         <v/>
       </c>
     </row>
+    <row r="1723"/>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
@@ -18734,6 +18832,8 @@
         <v/>
       </c>
     </row>
+    <row r="1728"/>
+    <row r="1729"/>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
@@ -19191,6 +19291,7 @@
         <v/>
       </c>
     </row>
+    <row r="1773"/>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
@@ -19244,6 +19345,8 @@
         <v/>
       </c>
     </row>
+    <row r="1778"/>
+    <row r="1779"/>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
@@ -19449,6 +19552,7 @@
         <v/>
       </c>
     </row>
+    <row r="1799"/>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
@@ -19502,6 +19606,8 @@
         <v/>
       </c>
     </row>
+    <row r="1804"/>
+    <row r="1805"/>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
@@ -19770,6 +19876,7 @@
         <v/>
       </c>
     </row>
+    <row r="1831"/>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
@@ -19823,6 +19930,8 @@
         <v/>
       </c>
     </row>
+    <row r="1836"/>
+    <row r="1837"/>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
@@ -20049,6 +20158,7 @@
         <v/>
       </c>
     </row>
+    <row r="1859"/>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
@@ -20102,6 +20212,8 @@
         <v/>
       </c>
     </row>
+    <row r="1864"/>
+    <row r="1865"/>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
@@ -20407,6 +20519,7 @@
         <v/>
       </c>
     </row>
+    <row r="1894"/>
     <row r="1895">
       <c r="A1895" t="inlineStr">
         <is>
@@ -20460,6 +20573,7 @@
         <v/>
       </c>
     </row>
+    <row r="1899"/>
     <row r="1900">
       <c r="A1900" t="inlineStr">
         <is>
@@ -20623,6 +20737,7 @@
         <v/>
       </c>
     </row>
+    <row r="1915"/>
     <row r="1916">
       <c r="A1916" t="inlineStr">
         <is>
@@ -21009,6 +21124,8 @@
       </c>
       <c r="D1947" s="40" t="n"/>
     </row>
+    <row r="1948"/>
+    <row r="1949"/>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
@@ -21151,6 +21268,7 @@
         <v/>
       </c>
     </row>
+    <row r="1963"/>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
@@ -21204,6 +21322,8 @@
         <v/>
       </c>
     </row>
+    <row r="1968"/>
+    <row r="1969"/>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
@@ -21388,6 +21508,7 @@
         <v/>
       </c>
     </row>
+    <row r="1987"/>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
@@ -21441,6 +21562,8 @@
         <v/>
       </c>
     </row>
+    <row r="1992"/>
+    <row r="1993"/>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
@@ -21922,6 +22045,7 @@
         <v/>
       </c>
     </row>
+    <row r="2039"/>
     <row r="2040">
       <c r="A2040" t="inlineStr">
         <is>
@@ -21975,6 +22099,7 @@
         <v/>
       </c>
     </row>
+    <row r="2044"/>
     <row r="2045">
       <c r="A2045" t="inlineStr">
         <is>
@@ -21997,6 +22122,8 @@
         <v>-75360.2</v>
       </c>
     </row>
+    <row r="2047"/>
+    <row r="2048"/>
     <row r="2049">
       <c r="A2049" t="inlineStr">
         <is>
@@ -22391,6 +22518,7 @@
         <v/>
       </c>
     </row>
+    <row r="2086"/>
     <row r="2087">
       <c r="A2087" t="inlineStr">
         <is>
@@ -22444,6 +22572,8 @@
         <v/>
       </c>
     </row>
+    <row r="2091"/>
+    <row r="2092"/>
     <row r="2093">
       <c r="A2093" t="inlineStr">
         <is>
@@ -22565,6 +22695,7 @@
         <v/>
       </c>
     </row>
+    <row r="2104"/>
     <row r="2105">
       <c r="A2105" t="inlineStr">
         <is>
@@ -22618,6 +22749,8 @@
         <v/>
       </c>
     </row>
+    <row r="2109"/>
+    <row r="2110"/>
     <row r="2111">
       <c r="A2111" t="inlineStr">
         <is>
@@ -22886,6 +23019,7 @@
         <v/>
       </c>
     </row>
+    <row r="2136"/>
     <row r="2137">
       <c r="A2137" t="inlineStr">
         <is>
@@ -22939,6 +23073,8 @@
         <v/>
       </c>
     </row>
+    <row r="2141"/>
+    <row r="2142"/>
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
@@ -23186,6 +23322,7 @@
         <v/>
       </c>
     </row>
+    <row r="2166"/>
     <row r="2167">
       <c r="A2167" t="inlineStr">
         <is>
@@ -23239,6 +23376,8 @@
         <v/>
       </c>
     </row>
+    <row r="2171"/>
+    <row r="2172"/>
     <row r="2173">
       <c r="A2173" t="inlineStr">
         <is>
@@ -23444,6 +23583,7 @@
         <v/>
       </c>
     </row>
+    <row r="2192"/>
     <row r="2193">
       <c r="A2193" t="inlineStr">
         <is>
@@ -23497,6 +23637,8 @@
         <v/>
       </c>
     </row>
+    <row r="2197"/>
+    <row r="2198"/>
     <row r="2199">
       <c r="A2199" t="inlineStr">
         <is>
@@ -23681,6 +23823,7 @@
         <v/>
       </c>
     </row>
+    <row r="2216"/>
     <row r="2217">
       <c r="A2217" t="inlineStr">
         <is>
@@ -23734,6 +23877,8 @@
         <v/>
       </c>
     </row>
+    <row r="2221"/>
+    <row r="2222"/>
     <row r="2223">
       <c r="A2223" t="inlineStr">
         <is>
@@ -23876,6 +24021,7 @@
         <v/>
       </c>
     </row>
+    <row r="2236"/>
     <row r="2237">
       <c r="A2237" t="inlineStr">
         <is>
@@ -23929,6 +24075,8 @@
         <v/>
       </c>
     </row>
+    <row r="2241"/>
+    <row r="2242"/>
     <row r="2243">
       <c r="A2243" t="inlineStr">
         <is>
@@ -24197,6 +24345,7 @@
         <v/>
       </c>
     </row>
+    <row r="2268"/>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
@@ -24250,6 +24399,8 @@
         <v/>
       </c>
     </row>
+    <row r="2273"/>
+    <row r="2274"/>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
@@ -24560,6 +24711,7 @@
         <v/>
       </c>
     </row>
+    <row r="2304"/>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
@@ -24613,6 +24765,8 @@
         <v/>
       </c>
     </row>
+    <row r="2309"/>
+    <row r="2310"/>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
@@ -24797,6 +24951,7 @@
         <v/>
       </c>
     </row>
+    <row r="2328"/>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
@@ -24850,6 +25005,8 @@
         <v/>
       </c>
     </row>
+    <row r="2333"/>
+    <row r="2334"/>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
@@ -25076,6 +25233,7 @@
         <v/>
       </c>
     </row>
+    <row r="2356"/>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
@@ -25129,6 +25287,7 @@
         <v/>
       </c>
     </row>
+    <row r="2361"/>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
@@ -25152,6 +25311,8 @@
         <v/>
       </c>
     </row>
+    <row r="2364"/>
+    <row r="2365"/>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
@@ -25198,6 +25359,7 @@
         <v/>
       </c>
     </row>
+    <row r="2370"/>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
@@ -25250,6 +25412,8 @@
         <v/>
       </c>
     </row>
+    <row r="2375"/>
+    <row r="2376"/>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
@@ -25413,6 +25577,7 @@
         <v/>
       </c>
     </row>
+    <row r="2392"/>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
@@ -25466,6 +25631,8 @@
         <v/>
       </c>
     </row>
+    <row r="2397"/>
+    <row r="2398"/>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
@@ -25755,6 +25922,7 @@
         <v/>
       </c>
     </row>
+    <row r="2426"/>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
@@ -25808,6 +25976,8 @@
         <v/>
       </c>
     </row>
+    <row r="2431"/>
+    <row r="2432"/>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
@@ -26202,6 +26372,7 @@
         <v/>
       </c>
     </row>
+    <row r="2470"/>
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
@@ -26255,6 +26426,8 @@
         <v/>
       </c>
     </row>
+    <row r="2475"/>
+    <row r="2476"/>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
@@ -26481,6 +26654,7 @@
         <v/>
       </c>
     </row>
+    <row r="2498"/>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
@@ -26534,6 +26708,8 @@
         <v/>
       </c>
     </row>
+    <row r="2503"/>
+    <row r="2504"/>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
@@ -26844,6 +27020,7 @@
         <v/>
       </c>
     </row>
+    <row r="2534"/>
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
@@ -26897,6 +27074,8 @@
         <v/>
       </c>
     </row>
+    <row r="2539"/>
+    <row r="2540"/>
     <row r="2541">
       <c r="A2541" t="inlineStr">
         <is>
@@ -26943,6 +27122,7 @@
         <v/>
       </c>
     </row>
+    <row r="2545"/>
     <row r="2546">
       <c r="A2546" t="inlineStr">
         <is>
@@ -26965,6 +27145,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2548"/>
+    <row r="2549"/>
     <row r="2550">
       <c r="A2550" t="inlineStr">
         <is>
@@ -27011,6 +27193,7 @@
         <v/>
       </c>
     </row>
+    <row r="2554"/>
     <row r="2555">
       <c r="A2555" t="inlineStr">
         <is>
@@ -27033,6 +27216,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2557"/>
+    <row r="2558"/>
     <row r="2559">
       <c r="A2559" t="inlineStr">
         <is>
@@ -27091,6 +27276,7 @@
         <v/>
       </c>
     </row>
+    <row r="2564"/>
     <row r="2565">
       <c r="A2565" t="inlineStr">
         <is>
@@ -27144,6 +27330,7 @@
         <v/>
       </c>
     </row>
+    <row r="2569"/>
     <row r="2570">
       <c r="A2570" t="inlineStr">
         <is>
@@ -27166,6 +27353,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2572"/>
+    <row r="2573"/>
     <row r="2574" s="44">
       <c r="A2574" t="inlineStr">
         <is>
@@ -27289,6 +27478,8 @@
         <v/>
       </c>
     </row>
+    <row r="2585"/>
+    <row r="2586"/>
     <row r="2587">
       <c r="A2587" t="inlineStr">
         <is>
@@ -27335,6 +27526,7 @@
         <v/>
       </c>
     </row>
+    <row r="2591"/>
     <row r="2592">
       <c r="A2592" t="inlineStr">
         <is>
@@ -27357,6 +27549,8 @@
         <v>-76610.5</v>
       </c>
     </row>
+    <row r="2594"/>
+    <row r="2595"/>
     <row r="2596">
       <c r="A2596" t="inlineStr">
         <is>
@@ -27403,6 +27597,8 @@
         <v/>
       </c>
     </row>
+    <row r="2600"/>
+    <row r="2601"/>
     <row r="2602">
       <c r="A2602" t="inlineStr">
         <is>
@@ -27482,6 +27678,7 @@
         <v/>
       </c>
     </row>
+    <row r="2609"/>
     <row r="2610">
       <c r="A2610" t="inlineStr">
         <is>
@@ -27535,6 +27732,7 @@
         <v/>
       </c>
     </row>
+    <row r="2614"/>
     <row r="2615">
       <c r="A2615" t="inlineStr">
         <is>
@@ -27595,6 +27793,8 @@
         <v/>
       </c>
     </row>
+    <row r="2620"/>
+    <row r="2621"/>
     <row r="2622">
       <c r="A2622" t="inlineStr">
         <is>
@@ -27680,6 +27880,7 @@
         <v/>
       </c>
     </row>
+    <row r="2630"/>
     <row r="2631">
       <c r="A2631" t="inlineStr">
         <is>
@@ -27733,56 +27934,190 @@
         <v/>
       </c>
     </row>
-    <row r="2636">
-      <c r="A2636" t="inlineStr">
-        <is>
-          <t>累積留倉   300股</t>
-        </is>
-      </c>
-    </row>
     <row r="2637">
       <c r="A2637" t="inlineStr">
         <is>
+          <t>2026.10.19</t>
+        </is>
+      </c>
+      <c r="B2637" t="n">
+        <v>2382582.4</v>
+      </c>
+      <c r="C2637" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2638">
+      <c r="A2638" t="n">
+        <v>76904.62</v>
+      </c>
+      <c r="B2638">
+        <f>+B2637+A2638</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" t="n">
+        <v>76911.58</v>
+      </c>
+      <c r="B2639">
+        <f>+B2638+A2639</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2640">
+      <c r="A2640" t="n">
+        <v>76973.91</v>
+      </c>
+      <c r="B2640">
+        <f>+B2639+A2640</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2641">
+      <c r="B2641" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2641" s="80">
+        <f>SUM(C2638:C2640)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2642">
+      <c r="B2642" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2642" s="80">
+        <f>+B2640-B2637-A2638-A2639-A2640</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2644">
+      <c r="A2644" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2645">
+      <c r="A2645" t="inlineStr">
+        <is>
           <t>2026.10.16 留倉</t>
         </is>
       </c>
-      <c r="B2637" t="inlineStr">
+      <c r="B2645" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2637" t="n">
+      <c r="C2645" t="n">
         <v>-76663.96000000001</v>
       </c>
     </row>
-    <row r="2638">
-      <c r="A2638" t="inlineStr">
+    <row r="2646">
+      <c r="A2646" t="inlineStr">
         <is>
           <t>2026.10.16 留倉</t>
         </is>
       </c>
-      <c r="B2638" t="inlineStr">
+      <c r="B2646" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2638" t="n">
+      <c r="C2646" t="n">
         <v>-76592.61</v>
       </c>
     </row>
-    <row r="2639">
-      <c r="A2639" t="inlineStr">
+    <row r="2647">
+      <c r="A2647" t="inlineStr">
         <is>
           <t>2026.10.16 留倉</t>
         </is>
       </c>
-      <c r="B2639" t="inlineStr">
+      <c r="B2647" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2639" t="n">
+      <c r="C2647" t="n">
         <v>-76401</v>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="A2648" t="inlineStr">
+        <is>
+          <t>2026.10.19 平倉</t>
+        </is>
+      </c>
+      <c r="B2648" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2648">
+        <f>+A2640</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="A2649" t="inlineStr">
+        <is>
+          <t>2026.10.19 平倉</t>
+        </is>
+      </c>
+      <c r="B2649" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2649">
+        <f>+A2639</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2650">
+      <c r="A2650" t="inlineStr">
+        <is>
+          <t>2026.10.19 平倉</t>
+        </is>
+      </c>
+      <c r="B2650" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2650">
+        <f>+A2638</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="B2651" t="inlineStr">
+        <is>
+          <t>平倉損益</t>
+        </is>
+      </c>
+      <c r="C2651">
+        <f>C2645+C2646+C2647+C2648+C2649+C2650</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="B2652" t="inlineStr">
+        <is>
+          <t>平倉損益 %</t>
+        </is>
+      </c>
+      <c r="C2652">
+        <f>C2651/ABS(C2645+C2646+C2647)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -27797,7 +28132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -28647,6 +28982,18 @@
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="86" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1132.54</v>
+      </c>
+      <c r="C71">
+        <f>C70+B71</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-22 10:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2652"/>
+  <dimension ref="A1:E2664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -27934,6 +27934,8 @@
         <v/>
       </c>
     </row>
+    <row r="2635"/>
+    <row r="2636"/>
     <row r="2637">
       <c r="A2637" t="inlineStr">
         <is>
@@ -27998,124 +28000,238 @@
         <v/>
       </c>
     </row>
-    <row r="2644">
-      <c r="A2644" t="inlineStr">
-        <is>
-          <t>累積留倉   0股</t>
-        </is>
-      </c>
-    </row>
+    <row r="2643"/>
+    <row r="2644"/>
     <row r="2645">
       <c r="A2645" t="inlineStr">
         <is>
+          <t>2026.10.21</t>
+        </is>
+      </c>
+      <c r="B2645" t="n">
+        <v>2383728.23</v>
+      </c>
+      <c r="C2645" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2646">
+      <c r="A2646" t="n">
+        <v>-77034.99000000001</v>
+      </c>
+      <c r="B2646">
+        <f>+B2645+A2646</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2647">
+      <c r="A2647" t="n">
+        <v>76893.42</v>
+      </c>
+      <c r="B2647">
+        <f>+B2646+A2647</f>
+        <v/>
+      </c>
+      <c r="C2647" t="n">
+        <v>-141.57</v>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="B2648" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2648" s="80">
+        <f>SUM(C2646:C2647)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="B2649" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2649" s="80">
+        <f>+B2647-B2645</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="A2651" t="inlineStr">
+        <is>
+          <t>2026.10.21當沖</t>
+        </is>
+      </c>
+      <c r="B2651" t="inlineStr">
+        <is>
+          <t>買</t>
+        </is>
+      </c>
+      <c r="C2651" s="80">
+        <f>SUMIF(A2646:A2647,"&lt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="A2652">
+        <f>"SPY " &amp; COUNT(C2646:C2647) * 100 &amp; "股"</f>
+        <v/>
+      </c>
+      <c r="B2652" t="inlineStr">
+        <is>
+          <t>賣</t>
+        </is>
+      </c>
+      <c r="C2652" s="80">
+        <f>SUMIF(A2646:A2647,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2653">
+      <c r="B2653" t="inlineStr">
+        <is>
+          <t>當日損益</t>
+        </is>
+      </c>
+      <c r="C2653" s="80">
+        <f>+C2651+C2652</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2654">
+      <c r="B2654" t="inlineStr">
+        <is>
+          <t>當日損益 %</t>
+        </is>
+      </c>
+      <c r="C2654" s="45">
+        <f>C2653/ABS(C2651)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2655"/>
+    <row r="2656">
+      <c r="A2656" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2657">
+      <c r="A2657" t="inlineStr">
+        <is>
           <t>2026.10.16 留倉</t>
         </is>
       </c>
-      <c r="B2645" t="inlineStr">
+      <c r="B2657" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2645" t="n">
+      <c r="C2657" t="n">
         <v>-76663.96000000001</v>
       </c>
     </row>
-    <row r="2646">
-      <c r="A2646" t="inlineStr">
+    <row r="2658">
+      <c r="A2658" t="inlineStr">
         <is>
           <t>2026.10.16 留倉</t>
         </is>
       </c>
-      <c r="B2646" t="inlineStr">
+      <c r="B2658" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2646" t="n">
+      <c r="C2658" t="n">
         <v>-76592.61</v>
       </c>
     </row>
-    <row r="2647">
-      <c r="A2647" t="inlineStr">
+    <row r="2659">
+      <c r="A2659" t="inlineStr">
         <is>
           <t>2026.10.16 留倉</t>
         </is>
       </c>
-      <c r="B2647" t="inlineStr">
+      <c r="B2659" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2647" t="n">
+      <c r="C2659" t="n">
         <v>-76401</v>
       </c>
     </row>
-    <row r="2648">
-      <c r="A2648" t="inlineStr">
+    <row r="2660">
+      <c r="A2660" t="inlineStr">
         <is>
           <t>2026.10.19 平倉</t>
         </is>
       </c>
-      <c r="B2648" t="inlineStr">
+      <c r="B2660" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2648">
+      <c r="C2660">
         <f>+A2640</f>
         <v/>
       </c>
     </row>
-    <row r="2649">
-      <c r="A2649" t="inlineStr">
+    <row r="2661">
+      <c r="A2661" t="inlineStr">
         <is>
           <t>2026.10.19 平倉</t>
         </is>
       </c>
-      <c r="B2649" t="inlineStr">
+      <c r="B2661" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2649">
+      <c r="C2661">
         <f>+A2639</f>
         <v/>
       </c>
     </row>
-    <row r="2650">
-      <c r="A2650" t="inlineStr">
+    <row r="2662">
+      <c r="A2662" t="inlineStr">
         <is>
           <t>2026.10.19 平倉</t>
         </is>
       </c>
-      <c r="B2650" t="inlineStr">
+      <c r="B2662" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2650">
+      <c r="C2662">
         <f>+A2638</f>
         <v/>
       </c>
     </row>
-    <row r="2651">
-      <c r="B2651" t="inlineStr">
+    <row r="2663">
+      <c r="B2663" t="inlineStr">
         <is>
           <t>平倉損益</t>
         </is>
       </c>
-      <c r="C2651">
+      <c r="C2663">
         <f>C2645+C2646+C2647+C2648+C2649+C2650</f>
         <v/>
       </c>
     </row>
-    <row r="2652">
-      <c r="B2652" t="inlineStr">
+    <row r="2664">
+      <c r="B2664" t="inlineStr">
         <is>
           <t>平倉損益 %</t>
         </is>
       </c>
-      <c r="C2652">
+      <c r="C2664">
         <f>C2651/ABS(C2645+C2646+C2647)</f>
         <v/>
       </c>
@@ -28132,7 +28248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -28994,6 +29110,18 @@
         <v/>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="86" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-141.57</v>
+      </c>
+      <c r="C72">
+        <f>C71+B72</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-22 12:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2664"/>
+  <dimension ref="A1:D2664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -11266,8 +11266,6 @@
         <v/>
       </c>
     </row>
-    <row r="975"/>
-    <row r="976"/>
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
@@ -11464,7 +11462,6 @@
         <v/>
       </c>
     </row>
-    <row r="996"/>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
@@ -11518,8 +11515,6 @@
         <v/>
       </c>
     </row>
-    <row r="1001"/>
-    <row r="1002"/>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
@@ -11559,8 +11554,6 @@
         <v/>
       </c>
     </row>
-    <row r="1006"/>
-    <row r="1007"/>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
@@ -11682,7 +11675,6 @@
         <v/>
       </c>
     </row>
-    <row r="1019"/>
     <row r="1020">
       <c r="A1020" t="inlineStr">
         <is>
@@ -11736,8 +11728,6 @@
         <v/>
       </c>
     </row>
-    <row r="1024"/>
-    <row r="1025"/>
     <row r="1026">
       <c r="A1026" t="inlineStr">
         <is>
@@ -11777,8 +11767,6 @@
         <v/>
       </c>
     </row>
-    <row r="1029"/>
-    <row r="1030"/>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
@@ -11840,7 +11828,6 @@
         <v/>
       </c>
     </row>
-    <row r="1036"/>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
@@ -11848,7 +11835,6 @@
         </is>
       </c>
     </row>
-    <row r="1038"/>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
@@ -11903,7 +11889,6 @@
         <v/>
       </c>
     </row>
-    <row r="1043"/>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
@@ -11958,7 +11943,6 @@
         <v/>
       </c>
     </row>
-    <row r="1048"/>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
@@ -12080,7 +12064,6 @@
         <v/>
       </c>
     </row>
-    <row r="1060"/>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
@@ -12134,8 +12117,6 @@
         <v/>
       </c>
     </row>
-    <row r="1065"/>
-    <row r="1066"/>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
@@ -12266,7 +12247,6 @@
         <v/>
       </c>
     </row>
-    <row r="1079"/>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
@@ -12320,7 +12300,6 @@
         <v/>
       </c>
     </row>
-    <row r="1084"/>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
@@ -12343,8 +12322,6 @@
         <v>-75037.94</v>
       </c>
     </row>
-    <row r="1087"/>
-    <row r="1088"/>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
@@ -12496,7 +12473,6 @@
         <v/>
       </c>
     </row>
-    <row r="1103"/>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
@@ -12550,7 +12526,6 @@
         <v/>
       </c>
     </row>
-    <row r="1108"/>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
@@ -12604,8 +12579,6 @@
         <v/>
       </c>
     </row>
-    <row r="1113"/>
-    <row r="1114"/>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
@@ -12706,7 +12679,6 @@
         <v/>
       </c>
     </row>
-    <row r="1124"/>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
@@ -12760,8 +12732,6 @@
         <v/>
       </c>
     </row>
-    <row r="1129"/>
-    <row r="1130"/>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
@@ -12925,7 +12895,6 @@
         <v/>
       </c>
     </row>
-    <row r="1146"/>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
@@ -12979,8 +12948,6 @@
         <v/>
       </c>
     </row>
-    <row r="1151"/>
-    <row r="1152"/>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
@@ -13144,7 +13111,6 @@
         <v/>
       </c>
     </row>
-    <row r="1168"/>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
@@ -13198,8 +13164,6 @@
         <v/>
       </c>
     </row>
-    <row r="1173"/>
-    <row r="1174"/>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
@@ -13369,7 +13333,6 @@
         <v/>
       </c>
     </row>
-    <row r="1191"/>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
@@ -13423,7 +13386,6 @@
         <v/>
       </c>
     </row>
-    <row r="1196"/>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
@@ -13476,8 +13438,6 @@
         <v>-74653</v>
       </c>
     </row>
-    <row r="1201"/>
-    <row r="1202"/>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
@@ -13608,7 +13568,6 @@
         <v/>
       </c>
     </row>
-    <row r="1215"/>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
@@ -13662,7 +13621,6 @@
         <v/>
       </c>
     </row>
-    <row r="1220"/>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
@@ -13716,7 +13674,6 @@
         <v/>
       </c>
     </row>
-    <row r="1225"/>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
@@ -13756,8 +13713,6 @@
         <v/>
       </c>
     </row>
-    <row r="1229"/>
-    <row r="1230"/>
     <row r="1231">
       <c r="A1231" s="80" t="inlineStr">
         <is>
@@ -14089,7 +14044,6 @@
         <v/>
       </c>
     </row>
-    <row r="1261"/>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
@@ -14143,7 +14097,6 @@
         <v/>
       </c>
     </row>
-    <row r="1266"/>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
@@ -14198,8 +14151,6 @@
         <v>-74291.5</v>
       </c>
     </row>
-    <row r="1271"/>
-    <row r="1272"/>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
@@ -14531,7 +14482,6 @@
         <v/>
       </c>
     </row>
-    <row r="1305"/>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
@@ -14585,7 +14535,6 @@
         <v/>
       </c>
     </row>
-    <row r="1310"/>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
@@ -14641,8 +14590,6 @@
         <v/>
       </c>
     </row>
-    <row r="1315"/>
-    <row r="1316"/>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
@@ -14878,7 +14825,6 @@
         <v/>
       </c>
     </row>
-    <row r="1339"/>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
@@ -14932,7 +14878,6 @@
         <v/>
       </c>
     </row>
-    <row r="1344"/>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
@@ -15003,7 +14948,6 @@
         <v>-72794.59</v>
       </c>
     </row>
-    <row r="1350"/>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
@@ -15188,7 +15132,6 @@
         <v/>
       </c>
     </row>
-    <row r="1368"/>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
@@ -15242,7 +15185,6 @@
         <v/>
       </c>
     </row>
-    <row r="1373"/>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
@@ -15314,7 +15256,6 @@
         <v/>
       </c>
     </row>
-    <row r="1379"/>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
@@ -15430,7 +15371,6 @@
         <v/>
       </c>
     </row>
-    <row r="1391"/>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
@@ -15484,7 +15424,6 @@
         <v/>
       </c>
     </row>
-    <row r="1396"/>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
@@ -15534,7 +15473,6 @@
         <v/>
       </c>
     </row>
-    <row r="1401"/>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
@@ -15584,7 +15522,6 @@
         <v/>
       </c>
     </row>
-    <row r="1406"/>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
@@ -15634,7 +15571,6 @@
         <v/>
       </c>
     </row>
-    <row r="1411"/>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
@@ -15684,8 +15620,6 @@
         <v/>
       </c>
     </row>
-    <row r="1416"/>
-    <row r="1417"/>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
@@ -15858,7 +15792,6 @@
         <v/>
       </c>
     </row>
-    <row r="1434"/>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
@@ -15915,7 +15848,6 @@
         <v/>
       </c>
     </row>
-    <row r="1439"/>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
@@ -15938,7 +15870,6 @@
         <v>-75313</v>
       </c>
     </row>
-    <row r="1442"/>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
@@ -16291,7 +16222,6 @@
         <v/>
       </c>
     </row>
-    <row r="1476"/>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
@@ -16345,8 +16275,6 @@
         <v/>
       </c>
     </row>
-    <row r="1481"/>
-    <row r="1482"/>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
@@ -16552,7 +16480,6 @@
         <v/>
       </c>
     </row>
-    <row r="1502"/>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
@@ -16606,8 +16533,6 @@
         <v/>
       </c>
     </row>
-    <row r="1507"/>
-    <row r="1508"/>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
@@ -16792,7 +16717,6 @@
         <v/>
       </c>
     </row>
-    <row r="1526"/>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
@@ -16846,8 +16770,6 @@
         <v/>
       </c>
     </row>
-    <row r="1531"/>
-    <row r="1532"/>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
@@ -17053,7 +16975,6 @@
         <v/>
       </c>
     </row>
-    <row r="1552"/>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
@@ -17107,8 +17028,6 @@
         <v/>
       </c>
     </row>
-    <row r="1557"/>
-    <row r="1558"/>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
@@ -17398,7 +17317,6 @@
         <v/>
       </c>
     </row>
-    <row r="1586"/>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
@@ -17452,7 +17370,6 @@
         <v/>
       </c>
     </row>
-    <row r="1591"/>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
@@ -17506,8 +17423,6 @@
         <v/>
       </c>
     </row>
-    <row r="1596"/>
-    <row r="1597"/>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
@@ -17671,7 +17586,6 @@
         <v/>
       </c>
     </row>
-    <row r="1613"/>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
@@ -17725,8 +17639,6 @@
         <v/>
       </c>
     </row>
-    <row r="1618"/>
-    <row r="1619"/>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
@@ -17995,7 +17907,6 @@
         <v/>
       </c>
     </row>
-    <row r="1645"/>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
@@ -18049,8 +17960,6 @@
         <v/>
       </c>
     </row>
-    <row r="1650"/>
-    <row r="1651"/>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
@@ -18277,7 +18186,6 @@
         <v/>
       </c>
     </row>
-    <row r="1673"/>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
@@ -18331,8 +18239,6 @@
         <v/>
       </c>
     </row>
-    <row r="1678"/>
-    <row r="1679"/>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
@@ -18496,7 +18402,6 @@
         <v/>
       </c>
     </row>
-    <row r="1695"/>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
@@ -18550,8 +18455,6 @@
         <v/>
       </c>
     </row>
-    <row r="1700"/>
-    <row r="1701"/>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
@@ -18778,7 +18681,6 @@
         <v/>
       </c>
     </row>
-    <row r="1723"/>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
@@ -18832,8 +18734,6 @@
         <v/>
       </c>
     </row>
-    <row r="1728"/>
-    <row r="1729"/>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
@@ -19291,7 +19191,6 @@
         <v/>
       </c>
     </row>
-    <row r="1773"/>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
@@ -19345,8 +19244,6 @@
         <v/>
       </c>
     </row>
-    <row r="1778"/>
-    <row r="1779"/>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
@@ -19552,7 +19449,6 @@
         <v/>
       </c>
     </row>
-    <row r="1799"/>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
@@ -19606,8 +19502,6 @@
         <v/>
       </c>
     </row>
-    <row r="1804"/>
-    <row r="1805"/>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
@@ -19876,7 +19770,6 @@
         <v/>
       </c>
     </row>
-    <row r="1831"/>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
@@ -19930,8 +19823,6 @@
         <v/>
       </c>
     </row>
-    <row r="1836"/>
-    <row r="1837"/>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
@@ -20158,7 +20049,6 @@
         <v/>
       </c>
     </row>
-    <row r="1859"/>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
@@ -20212,8 +20102,6 @@
         <v/>
       </c>
     </row>
-    <row r="1864"/>
-    <row r="1865"/>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
@@ -20519,7 +20407,6 @@
         <v/>
       </c>
     </row>
-    <row r="1894"/>
     <row r="1895">
       <c r="A1895" t="inlineStr">
         <is>
@@ -20573,7 +20460,6 @@
         <v/>
       </c>
     </row>
-    <row r="1899"/>
     <row r="1900">
       <c r="A1900" t="inlineStr">
         <is>
@@ -20737,7 +20623,6 @@
         <v/>
       </c>
     </row>
-    <row r="1915"/>
     <row r="1916">
       <c r="A1916" t="inlineStr">
         <is>
@@ -21124,8 +21009,6 @@
       </c>
       <c r="D1947" s="40" t="n"/>
     </row>
-    <row r="1948"/>
-    <row r="1949"/>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
@@ -21268,7 +21151,6 @@
         <v/>
       </c>
     </row>
-    <row r="1963"/>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
@@ -21322,8 +21204,6 @@
         <v/>
       </c>
     </row>
-    <row r="1968"/>
-    <row r="1969"/>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
@@ -21508,7 +21388,6 @@
         <v/>
       </c>
     </row>
-    <row r="1987"/>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
@@ -21562,8 +21441,6 @@
         <v/>
       </c>
     </row>
-    <row r="1992"/>
-    <row r="1993"/>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
@@ -22045,7 +21922,6 @@
         <v/>
       </c>
     </row>
-    <row r="2039"/>
     <row r="2040">
       <c r="A2040" t="inlineStr">
         <is>
@@ -22099,7 +21975,6 @@
         <v/>
       </c>
     </row>
-    <row r="2044"/>
     <row r="2045">
       <c r="A2045" t="inlineStr">
         <is>
@@ -22122,8 +21997,6 @@
         <v>-75360.2</v>
       </c>
     </row>
-    <row r="2047"/>
-    <row r="2048"/>
     <row r="2049">
       <c r="A2049" t="inlineStr">
         <is>
@@ -22518,7 +22391,6 @@
         <v/>
       </c>
     </row>
-    <row r="2086"/>
     <row r="2087">
       <c r="A2087" t="inlineStr">
         <is>
@@ -22572,8 +22444,6 @@
         <v/>
       </c>
     </row>
-    <row r="2091"/>
-    <row r="2092"/>
     <row r="2093">
       <c r="A2093" t="inlineStr">
         <is>
@@ -22695,7 +22565,6 @@
         <v/>
       </c>
     </row>
-    <row r="2104"/>
     <row r="2105">
       <c r="A2105" t="inlineStr">
         <is>
@@ -22749,8 +22618,6 @@
         <v/>
       </c>
     </row>
-    <row r="2109"/>
-    <row r="2110"/>
     <row r="2111">
       <c r="A2111" t="inlineStr">
         <is>
@@ -23019,7 +22886,6 @@
         <v/>
       </c>
     </row>
-    <row r="2136"/>
     <row r="2137">
       <c r="A2137" t="inlineStr">
         <is>
@@ -23073,8 +22939,6 @@
         <v/>
       </c>
     </row>
-    <row r="2141"/>
-    <row r="2142"/>
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
@@ -23322,7 +23186,6 @@
         <v/>
       </c>
     </row>
-    <row r="2166"/>
     <row r="2167">
       <c r="A2167" t="inlineStr">
         <is>
@@ -23376,8 +23239,6 @@
         <v/>
       </c>
     </row>
-    <row r="2171"/>
-    <row r="2172"/>
     <row r="2173">
       <c r="A2173" t="inlineStr">
         <is>
@@ -23583,7 +23444,6 @@
         <v/>
       </c>
     </row>
-    <row r="2192"/>
     <row r="2193">
       <c r="A2193" t="inlineStr">
         <is>
@@ -23637,8 +23497,6 @@
         <v/>
       </c>
     </row>
-    <row r="2197"/>
-    <row r="2198"/>
     <row r="2199">
       <c r="A2199" t="inlineStr">
         <is>
@@ -23823,7 +23681,6 @@
         <v/>
       </c>
     </row>
-    <row r="2216"/>
     <row r="2217">
       <c r="A2217" t="inlineStr">
         <is>
@@ -23877,8 +23734,6 @@
         <v/>
       </c>
     </row>
-    <row r="2221"/>
-    <row r="2222"/>
     <row r="2223">
       <c r="A2223" t="inlineStr">
         <is>
@@ -24021,7 +23876,6 @@
         <v/>
       </c>
     </row>
-    <row r="2236"/>
     <row r="2237">
       <c r="A2237" t="inlineStr">
         <is>
@@ -24075,8 +23929,6 @@
         <v/>
       </c>
     </row>
-    <row r="2241"/>
-    <row r="2242"/>
     <row r="2243">
       <c r="A2243" t="inlineStr">
         <is>
@@ -24345,7 +24197,6 @@
         <v/>
       </c>
     </row>
-    <row r="2268"/>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
@@ -24399,8 +24250,6 @@
         <v/>
       </c>
     </row>
-    <row r="2273"/>
-    <row r="2274"/>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
@@ -24711,7 +24560,6 @@
         <v/>
       </c>
     </row>
-    <row r="2304"/>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
@@ -24765,8 +24613,6 @@
         <v/>
       </c>
     </row>
-    <row r="2309"/>
-    <row r="2310"/>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
@@ -24951,7 +24797,6 @@
         <v/>
       </c>
     </row>
-    <row r="2328"/>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
@@ -25005,8 +24850,6 @@
         <v/>
       </c>
     </row>
-    <row r="2333"/>
-    <row r="2334"/>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
@@ -25233,7 +25076,6 @@
         <v/>
       </c>
     </row>
-    <row r="2356"/>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
@@ -25287,7 +25129,6 @@
         <v/>
       </c>
     </row>
-    <row r="2361"/>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
@@ -25311,8 +25152,6 @@
         <v/>
       </c>
     </row>
-    <row r="2364"/>
-    <row r="2365"/>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
@@ -25359,7 +25198,6 @@
         <v/>
       </c>
     </row>
-    <row r="2370"/>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
@@ -25412,8 +25250,6 @@
         <v/>
       </c>
     </row>
-    <row r="2375"/>
-    <row r="2376"/>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
@@ -25577,7 +25413,6 @@
         <v/>
       </c>
     </row>
-    <row r="2392"/>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
@@ -25631,8 +25466,6 @@
         <v/>
       </c>
     </row>
-    <row r="2397"/>
-    <row r="2398"/>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
@@ -25922,7 +25755,6 @@
         <v/>
       </c>
     </row>
-    <row r="2426"/>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
@@ -25976,8 +25808,6 @@
         <v/>
       </c>
     </row>
-    <row r="2431"/>
-    <row r="2432"/>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
@@ -26372,7 +26202,6 @@
         <v/>
       </c>
     </row>
-    <row r="2470"/>
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
@@ -26426,8 +26255,6 @@
         <v/>
       </c>
     </row>
-    <row r="2475"/>
-    <row r="2476"/>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
@@ -26654,7 +26481,6 @@
         <v/>
       </c>
     </row>
-    <row r="2498"/>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
@@ -26708,8 +26534,6 @@
         <v/>
       </c>
     </row>
-    <row r="2503"/>
-    <row r="2504"/>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
@@ -27020,7 +26844,6 @@
         <v/>
       </c>
     </row>
-    <row r="2534"/>
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
@@ -27074,8 +26897,6 @@
         <v/>
       </c>
     </row>
-    <row r="2539"/>
-    <row r="2540"/>
     <row r="2541">
       <c r="A2541" t="inlineStr">
         <is>
@@ -27122,7 +26943,6 @@
         <v/>
       </c>
     </row>
-    <row r="2545"/>
     <row r="2546">
       <c r="A2546" t="inlineStr">
         <is>
@@ -27145,8 +26965,6 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2548"/>
-    <row r="2549"/>
     <row r="2550">
       <c r="A2550" t="inlineStr">
         <is>
@@ -27193,7 +27011,6 @@
         <v/>
       </c>
     </row>
-    <row r="2554"/>
     <row r="2555">
       <c r="A2555" t="inlineStr">
         <is>
@@ -27216,8 +27033,6 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2557"/>
-    <row r="2558"/>
     <row r="2559">
       <c r="A2559" t="inlineStr">
         <is>
@@ -27276,7 +27091,6 @@
         <v/>
       </c>
     </row>
-    <row r="2564"/>
     <row r="2565">
       <c r="A2565" t="inlineStr">
         <is>
@@ -27330,7 +27144,6 @@
         <v/>
       </c>
     </row>
-    <row r="2569"/>
     <row r="2570">
       <c r="A2570" t="inlineStr">
         <is>
@@ -27353,8 +27166,6 @@
         <v>-75688.5</v>
       </c>
     </row>
-    <row r="2572"/>
-    <row r="2573"/>
     <row r="2574" s="44">
       <c r="A2574" t="inlineStr">
         <is>
@@ -27478,8 +27289,6 @@
         <v/>
       </c>
     </row>
-    <row r="2585"/>
-    <row r="2586"/>
     <row r="2587">
       <c r="A2587" t="inlineStr">
         <is>
@@ -27526,7 +27335,6 @@
         <v/>
       </c>
     </row>
-    <row r="2591"/>
     <row r="2592">
       <c r="A2592" t="inlineStr">
         <is>
@@ -27549,8 +27357,6 @@
         <v>-76610.5</v>
       </c>
     </row>
-    <row r="2594"/>
-    <row r="2595"/>
     <row r="2596">
       <c r="A2596" t="inlineStr">
         <is>
@@ -27597,8 +27403,6 @@
         <v/>
       </c>
     </row>
-    <row r="2600"/>
-    <row r="2601"/>
     <row r="2602">
       <c r="A2602" t="inlineStr">
         <is>
@@ -27678,7 +27482,6 @@
         <v/>
       </c>
     </row>
-    <row r="2609"/>
     <row r="2610">
       <c r="A2610" t="inlineStr">
         <is>
@@ -27732,7 +27535,6 @@
         <v/>
       </c>
     </row>
-    <row r="2614"/>
     <row r="2615">
       <c r="A2615" t="inlineStr">
         <is>
@@ -27793,8 +27595,6 @@
         <v/>
       </c>
     </row>
-    <row r="2620"/>
-    <row r="2621"/>
     <row r="2622">
       <c r="A2622" t="inlineStr">
         <is>
@@ -27880,7 +27680,6 @@
         <v/>
       </c>
     </row>
-    <row r="2630"/>
     <row r="2631">
       <c r="A2631" t="inlineStr">
         <is>
@@ -27934,8 +27733,6 @@
         <v/>
       </c>
     </row>
-    <row r="2635"/>
-    <row r="2636"/>
     <row r="2637">
       <c r="A2637" t="inlineStr">
         <is>
@@ -28000,8 +27797,6 @@
         <v/>
       </c>
     </row>
-    <row r="2643"/>
-    <row r="2644"/>
     <row r="2645">
       <c r="A2645" t="inlineStr">
         <is>
@@ -28113,7 +27908,6 @@
         <v/>
       </c>
     </row>
-    <row r="2655"/>
     <row r="2656">
       <c r="A2656" t="inlineStr">
         <is>
@@ -28221,7 +28015,7 @@
         </is>
       </c>
       <c r="C2663">
-        <f>C2645+C2646+C2647+C2648+C2649+C2650</f>
+        <f>C2657+C2658+C2659+C2660+C2661+C2662</f>
         <v/>
       </c>
     </row>
@@ -28232,7 +28026,7 @@
         </is>
       </c>
       <c r="C2664">
-        <f>C2651/ABS(C2645+C2646+C2647)</f>
+        <f>C2663/ABS(C2657+C2658+C2659)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
p502 sync 2026-10-27 10:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2664"/>
+  <dimension ref="A1:E2679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -11266,6 +11266,8 @@
         <v/>
       </c>
     </row>
+    <row r="975"/>
+    <row r="976"/>
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
@@ -11462,6 +11464,7 @@
         <v/>
       </c>
     </row>
+    <row r="996"/>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
@@ -11515,6 +11518,8 @@
         <v/>
       </c>
     </row>
+    <row r="1001"/>
+    <row r="1002"/>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
@@ -11554,6 +11559,8 @@
         <v/>
       </c>
     </row>
+    <row r="1006"/>
+    <row r="1007"/>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
@@ -11675,6 +11682,7 @@
         <v/>
       </c>
     </row>
+    <row r="1019"/>
     <row r="1020">
       <c r="A1020" t="inlineStr">
         <is>
@@ -11728,6 +11736,8 @@
         <v/>
       </c>
     </row>
+    <row r="1024"/>
+    <row r="1025"/>
     <row r="1026">
       <c r="A1026" t="inlineStr">
         <is>
@@ -11767,6 +11777,8 @@
         <v/>
       </c>
     </row>
+    <row r="1029"/>
+    <row r="1030"/>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
@@ -11828,6 +11840,7 @@
         <v/>
       </c>
     </row>
+    <row r="1036"/>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
@@ -11835,6 +11848,7 @@
         </is>
       </c>
     </row>
+    <row r="1038"/>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
@@ -11889,6 +11903,7 @@
         <v/>
       </c>
     </row>
+    <row r="1043"/>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
@@ -11943,6 +11958,7 @@
         <v/>
       </c>
     </row>
+    <row r="1048"/>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
@@ -12064,6 +12080,7 @@
         <v/>
       </c>
     </row>
+    <row r="1060"/>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
@@ -12117,6 +12134,8 @@
         <v/>
       </c>
     </row>
+    <row r="1065"/>
+    <row r="1066"/>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
@@ -12247,6 +12266,7 @@
         <v/>
       </c>
     </row>
+    <row r="1079"/>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
@@ -12300,6 +12320,7 @@
         <v/>
       </c>
     </row>
+    <row r="1084"/>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
@@ -12322,6 +12343,8 @@
         <v>-75037.94</v>
       </c>
     </row>
+    <row r="1087"/>
+    <row r="1088"/>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
@@ -12473,6 +12496,7 @@
         <v/>
       </c>
     </row>
+    <row r="1103"/>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
@@ -12526,6 +12550,7 @@
         <v/>
       </c>
     </row>
+    <row r="1108"/>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
@@ -12579,6 +12604,8 @@
         <v/>
       </c>
     </row>
+    <row r="1113"/>
+    <row r="1114"/>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
@@ -12679,6 +12706,7 @@
         <v/>
       </c>
     </row>
+    <row r="1124"/>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
@@ -12732,6 +12760,8 @@
         <v/>
       </c>
     </row>
+    <row r="1129"/>
+    <row r="1130"/>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
@@ -12895,6 +12925,7 @@
         <v/>
       </c>
     </row>
+    <row r="1146"/>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
@@ -12948,6 +12979,8 @@
         <v/>
       </c>
     </row>
+    <row r="1151"/>
+    <row r="1152"/>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
@@ -13111,6 +13144,7 @@
         <v/>
       </c>
     </row>
+    <row r="1168"/>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
@@ -13164,6 +13198,8 @@
         <v/>
       </c>
     </row>
+    <row r="1173"/>
+    <row r="1174"/>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
@@ -13333,6 +13369,7 @@
         <v/>
       </c>
     </row>
+    <row r="1191"/>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
@@ -13386,6 +13423,7 @@
         <v/>
       </c>
     </row>
+    <row r="1196"/>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
@@ -13438,6 +13476,8 @@
         <v>-74653</v>
       </c>
     </row>
+    <row r="1201"/>
+    <row r="1202"/>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
@@ -13568,6 +13608,7 @@
         <v/>
       </c>
     </row>
+    <row r="1215"/>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
@@ -13621,6 +13662,7 @@
         <v/>
       </c>
     </row>
+    <row r="1220"/>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
@@ -13674,6 +13716,7 @@
         <v/>
       </c>
     </row>
+    <row r="1225"/>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
@@ -13713,6 +13756,8 @@
         <v/>
       </c>
     </row>
+    <row r="1229"/>
+    <row r="1230"/>
     <row r="1231">
       <c r="A1231" s="80" t="inlineStr">
         <is>
@@ -14044,6 +14089,7 @@
         <v/>
       </c>
     </row>
+    <row r="1261"/>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
@@ -14097,6 +14143,7 @@
         <v/>
       </c>
     </row>
+    <row r="1266"/>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
@@ -14151,6 +14198,8 @@
         <v>-74291.5</v>
       </c>
     </row>
+    <row r="1271"/>
+    <row r="1272"/>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
@@ -14482,6 +14531,7 @@
         <v/>
       </c>
     </row>
+    <row r="1305"/>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
@@ -14535,6 +14585,7 @@
         <v/>
       </c>
     </row>
+    <row r="1310"/>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
@@ -14590,6 +14641,8 @@
         <v/>
       </c>
     </row>
+    <row r="1315"/>
+    <row r="1316"/>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
@@ -14825,6 +14878,7 @@
         <v/>
       </c>
     </row>
+    <row r="1339"/>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
@@ -14878,6 +14932,7 @@
         <v/>
       </c>
     </row>
+    <row r="1344"/>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
@@ -14948,6 +15003,7 @@
         <v>-72794.59</v>
       </c>
     </row>
+    <row r="1350"/>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
@@ -15132,6 +15188,7 @@
         <v/>
       </c>
     </row>
+    <row r="1368"/>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
@@ -15185,6 +15242,7 @@
         <v/>
       </c>
     </row>
+    <row r="1373"/>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
@@ -15256,6 +15314,7 @@
         <v/>
       </c>
     </row>
+    <row r="1379"/>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
@@ -15371,6 +15430,7 @@
         <v/>
       </c>
     </row>
+    <row r="1391"/>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
@@ -15424,6 +15484,7 @@
         <v/>
       </c>
     </row>
+    <row r="1396"/>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
@@ -15473,6 +15534,7 @@
         <v/>
       </c>
     </row>
+    <row r="1401"/>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
@@ -15522,6 +15584,7 @@
         <v/>
       </c>
     </row>
+    <row r="1406"/>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
@@ -15571,6 +15634,7 @@
         <v/>
       </c>
     </row>
+    <row r="1411"/>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
@@ -15620,6 +15684,8 @@
         <v/>
       </c>
     </row>
+    <row r="1416"/>
+    <row r="1417"/>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
@@ -15792,6 +15858,7 @@
         <v/>
       </c>
     </row>
+    <row r="1434"/>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
@@ -15848,6 +15915,7 @@
         <v/>
       </c>
     </row>
+    <row r="1439"/>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
@@ -15870,6 +15938,7 @@
         <v>-75313</v>
       </c>
     </row>
+    <row r="1442"/>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
@@ -16222,6 +16291,7 @@
         <v/>
       </c>
     </row>
+    <row r="1476"/>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
@@ -16275,6 +16345,8 @@
         <v/>
       </c>
     </row>
+    <row r="1481"/>
+    <row r="1482"/>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
@@ -16480,6 +16552,7 @@
         <v/>
       </c>
     </row>
+    <row r="1502"/>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
@@ -16533,6 +16606,8 @@
         <v/>
       </c>
     </row>
+    <row r="1507"/>
+    <row r="1508"/>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
@@ -16717,6 +16792,7 @@
         <v/>
       </c>
     </row>
+    <row r="1526"/>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
@@ -16770,6 +16846,8 @@
         <v/>
       </c>
     </row>
+    <row r="1531"/>
+    <row r="1532"/>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
@@ -16975,6 +17053,7 @@
         <v/>
       </c>
     </row>
+    <row r="1552"/>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
@@ -17028,6 +17107,8 @@
         <v/>
       </c>
     </row>
+    <row r="1557"/>
+    <row r="1558"/>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
@@ -17317,6 +17398,7 @@
         <v/>
       </c>
     </row>
+    <row r="1586"/>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
@@ -17370,6 +17452,7 @@
         <v/>
       </c>
     </row>
+    <row r="1591"/>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
@@ -17423,6 +17506,8 @@
         <v/>
       </c>
     </row>
+    <row r="1596"/>
+    <row r="1597"/>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
@@ -17586,6 +17671,7 @@
         <v/>
       </c>
     </row>
+    <row r="1613"/>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
@@ -17639,6 +17725,8 @@
         <v/>
       </c>
     </row>
+    <row r="1618"/>
+    <row r="1619"/>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
@@ -17907,6 +17995,7 @@
         <v/>
       </c>
     </row>
+    <row r="1645"/>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
@@ -17960,6 +18049,8 @@
         <v/>
       </c>
     </row>
+    <row r="1650"/>
+    <row r="1651"/>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
@@ -18186,6 +18277,7 @@
         <v/>
       </c>
     </row>
+    <row r="1673"/>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
@@ -18239,6 +18331,8 @@
         <v/>
       </c>
     </row>
+    <row r="1678"/>
+    <row r="1679"/>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
@@ -18402,6 +18496,7 @@
         <v/>
       </c>
     </row>
+    <row r="1695"/>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
@@ -18455,6 +18550,8 @@
         <v/>
       </c>
     </row>
+    <row r="1700"/>
+    <row r="1701"/>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
@@ -18681,6 +18778,7 @@
         <v/>
       </c>
     </row>
+    <row r="1723"/>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
@@ -18734,6 +18832,8 @@
         <v/>
       </c>
     </row>
+    <row r="1728"/>
+    <row r="1729"/>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
@@ -19191,6 +19291,7 @@
         <v/>
       </c>
     </row>
+    <row r="1773"/>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
@@ -19244,6 +19345,8 @@
         <v/>
       </c>
     </row>
+    <row r="1778"/>
+    <row r="1779"/>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
@@ -19449,6 +19552,7 @@
         <v/>
       </c>
     </row>
+    <row r="1799"/>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
@@ -19502,6 +19606,8 @@
         <v/>
       </c>
     </row>
+    <row r="1804"/>
+    <row r="1805"/>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
@@ -19770,6 +19876,7 @@
         <v/>
       </c>
     </row>
+    <row r="1831"/>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
@@ -19823,6 +19930,8 @@
         <v/>
       </c>
     </row>
+    <row r="1836"/>
+    <row r="1837"/>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
@@ -20049,6 +20158,7 @@
         <v/>
       </c>
     </row>
+    <row r="1859"/>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
@@ -20102,6 +20212,8 @@
         <v/>
       </c>
     </row>
+    <row r="1864"/>
+    <row r="1865"/>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
@@ -20407,6 +20519,7 @@
         <v/>
       </c>
     </row>
+    <row r="1894"/>
     <row r="1895">
       <c r="A1895" t="inlineStr">
         <is>
@@ -20460,6 +20573,7 @@
         <v/>
       </c>
     </row>
+    <row r="1899"/>
     <row r="1900">
       <c r="A1900" t="inlineStr">
         <is>
@@ -20623,6 +20737,7 @@
         <v/>
       </c>
     </row>
+    <row r="1915"/>
     <row r="1916">
       <c r="A1916" t="inlineStr">
         <is>
@@ -21009,6 +21124,8 @@
       </c>
       <c r="D1947" s="40" t="n"/>
     </row>
+    <row r="1948"/>
+    <row r="1949"/>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
@@ -21151,6 +21268,7 @@
         <v/>
       </c>
     </row>
+    <row r="1963"/>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
@@ -21204,6 +21322,8 @@
         <v/>
       </c>
     </row>
+    <row r="1968"/>
+    <row r="1969"/>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
@@ -21388,6 +21508,7 @@
         <v/>
       </c>
     </row>
+    <row r="1987"/>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
@@ -21441,6 +21562,8 @@
         <v/>
       </c>
     </row>
+    <row r="1992"/>
+    <row r="1993"/>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
@@ -21922,6 +22045,7 @@
         <v/>
       </c>
     </row>
+    <row r="2039"/>
     <row r="2040">
       <c r="A2040" t="inlineStr">
         <is>
@@ -21975,6 +22099,7 @@
         <v/>
       </c>
     </row>
+    <row r="2044"/>
     <row r="2045">
       <c r="A2045" t="inlineStr">
         <is>
@@ -21997,6 +22122,8 @@
         <v>-75360.2</v>
       </c>
     </row>
+    <row r="2047"/>
+    <row r="2048"/>
     <row r="2049">
       <c r="A2049" t="inlineStr">
         <is>
@@ -22391,6 +22518,7 @@
         <v/>
       </c>
     </row>
+    <row r="2086"/>
     <row r="2087">
       <c r="A2087" t="inlineStr">
         <is>
@@ -22444,6 +22572,8 @@
         <v/>
       </c>
     </row>
+    <row r="2091"/>
+    <row r="2092"/>
     <row r="2093">
       <c r="A2093" t="inlineStr">
         <is>
@@ -22565,6 +22695,7 @@
         <v/>
       </c>
     </row>
+    <row r="2104"/>
     <row r="2105">
       <c r="A2105" t="inlineStr">
         <is>
@@ -22618,6 +22749,8 @@
         <v/>
       </c>
     </row>
+    <row r="2109"/>
+    <row r="2110"/>
     <row r="2111">
       <c r="A2111" t="inlineStr">
         <is>
@@ -22886,6 +23019,7 @@
         <v/>
       </c>
     </row>
+    <row r="2136"/>
     <row r="2137">
       <c r="A2137" t="inlineStr">
         <is>
@@ -22939,6 +23073,8 @@
         <v/>
       </c>
     </row>
+    <row r="2141"/>
+    <row r="2142"/>
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
@@ -23186,6 +23322,7 @@
         <v/>
       </c>
     </row>
+    <row r="2166"/>
     <row r="2167">
       <c r="A2167" t="inlineStr">
         <is>
@@ -23239,6 +23376,8 @@
         <v/>
       </c>
     </row>
+    <row r="2171"/>
+    <row r="2172"/>
     <row r="2173">
       <c r="A2173" t="inlineStr">
         <is>
@@ -23444,6 +23583,7 @@
         <v/>
       </c>
     </row>
+    <row r="2192"/>
     <row r="2193">
       <c r="A2193" t="inlineStr">
         <is>
@@ -23497,6 +23637,8 @@
         <v/>
       </c>
     </row>
+    <row r="2197"/>
+    <row r="2198"/>
     <row r="2199">
       <c r="A2199" t="inlineStr">
         <is>
@@ -23681,6 +23823,7 @@
         <v/>
       </c>
     </row>
+    <row r="2216"/>
     <row r="2217">
       <c r="A2217" t="inlineStr">
         <is>
@@ -23734,6 +23877,8 @@
         <v/>
       </c>
     </row>
+    <row r="2221"/>
+    <row r="2222"/>
     <row r="2223">
       <c r="A2223" t="inlineStr">
         <is>
@@ -23876,6 +24021,7 @@
         <v/>
       </c>
     </row>
+    <row r="2236"/>
     <row r="2237">
       <c r="A2237" t="inlineStr">
         <is>
@@ -23929,6 +24075,8 @@
         <v/>
       </c>
     </row>
+    <row r="2241"/>
+    <row r="2242"/>
     <row r="2243">
       <c r="A2243" t="inlineStr">
         <is>
@@ -24197,6 +24345,7 @@
         <v/>
       </c>
     </row>
+    <row r="2268"/>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
@@ -24250,6 +24399,8 @@
         <v/>
       </c>
     </row>
+    <row r="2273"/>
+    <row r="2274"/>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
@@ -24560,6 +24711,7 @@
         <v/>
       </c>
     </row>
+    <row r="2304"/>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
@@ -24613,6 +24765,8 @@
         <v/>
       </c>
     </row>
+    <row r="2309"/>
+    <row r="2310"/>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
@@ -24797,6 +24951,7 @@
         <v/>
       </c>
     </row>
+    <row r="2328"/>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
@@ -24850,6 +25005,8 @@
         <v/>
       </c>
     </row>
+    <row r="2333"/>
+    <row r="2334"/>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
@@ -25076,6 +25233,7 @@
         <v/>
       </c>
     </row>
+    <row r="2356"/>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
@@ -25129,6 +25287,7 @@
         <v/>
       </c>
     </row>
+    <row r="2361"/>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
@@ -25152,6 +25311,8 @@
         <v/>
       </c>
     </row>
+    <row r="2364"/>
+    <row r="2365"/>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
@@ -25198,6 +25359,7 @@
         <v/>
       </c>
     </row>
+    <row r="2370"/>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
@@ -25250,6 +25412,8 @@
         <v/>
       </c>
     </row>
+    <row r="2375"/>
+    <row r="2376"/>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
@@ -25413,6 +25577,7 @@
         <v/>
       </c>
     </row>
+    <row r="2392"/>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
@@ -25466,6 +25631,8 @@
         <v/>
       </c>
     </row>
+    <row r="2397"/>
+    <row r="2398"/>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
@@ -25755,6 +25922,7 @@
         <v/>
       </c>
     </row>
+    <row r="2426"/>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
@@ -25808,6 +25976,8 @@
         <v/>
       </c>
     </row>
+    <row r="2431"/>
+    <row r="2432"/>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
@@ -26202,6 +26372,7 @@
         <v/>
       </c>
     </row>
+    <row r="2470"/>
     <row r="2471">
       <c r="A2471" t="inlineStr">
         <is>
@@ -26255,6 +26426,8 @@
         <v/>
       </c>
     </row>
+    <row r="2475"/>
+    <row r="2476"/>
     <row r="2477">
       <c r="A2477" t="inlineStr">
         <is>
@@ -26481,6 +26654,7 @@
         <v/>
       </c>
     </row>
+    <row r="2498"/>
     <row r="2499">
       <c r="A2499" t="inlineStr">
         <is>
@@ -26534,6 +26708,8 @@
         <v/>
       </c>
     </row>
+    <row r="2503"/>
+    <row r="2504"/>
     <row r="2505">
       <c r="A2505" t="inlineStr">
         <is>
@@ -26844,6 +27020,7 @@
         <v/>
       </c>
     </row>
+    <row r="2534"/>
     <row r="2535">
       <c r="A2535" t="inlineStr">
         <is>
@@ -26897,6 +27074,8 @@
         <v/>
       </c>
     </row>
+    <row r="2539"/>
+    <row r="2540"/>
     <row r="2541">
       <c r="A2541" t="inlineStr">
         <is>
@@ -26943,6 +27122,7 @@
         <v/>
       </c>
     </row>
+    <row r="2545"/>
     <row r="2546">
       <c r="A2546" t="inlineStr">
         <is>
@@ -26965,6 +27145,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2548"/>
+    <row r="2549"/>
     <row r="2550">
       <c r="A2550" t="inlineStr">
         <is>
@@ -27011,6 +27193,7 @@
         <v/>
       </c>
     </row>
+    <row r="2554"/>
     <row r="2555">
       <c r="A2555" t="inlineStr">
         <is>
@@ -27033,6 +27216,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2557"/>
+    <row r="2558"/>
     <row r="2559">
       <c r="A2559" t="inlineStr">
         <is>
@@ -27091,6 +27276,7 @@
         <v/>
       </c>
     </row>
+    <row r="2564"/>
     <row r="2565">
       <c r="A2565" t="inlineStr">
         <is>
@@ -27144,6 +27330,7 @@
         <v/>
       </c>
     </row>
+    <row r="2569"/>
     <row r="2570">
       <c r="A2570" t="inlineStr">
         <is>
@@ -27166,6 +27353,8 @@
         <v>-75688.5</v>
       </c>
     </row>
+    <row r="2572"/>
+    <row r="2573"/>
     <row r="2574" s="44">
       <c r="A2574" t="inlineStr">
         <is>
@@ -27289,6 +27478,8 @@
         <v/>
       </c>
     </row>
+    <row r="2585"/>
+    <row r="2586"/>
     <row r="2587">
       <c r="A2587" t="inlineStr">
         <is>
@@ -27335,6 +27526,7 @@
         <v/>
       </c>
     </row>
+    <row r="2591"/>
     <row r="2592">
       <c r="A2592" t="inlineStr">
         <is>
@@ -27357,6 +27549,8 @@
         <v>-76610.5</v>
       </c>
     </row>
+    <row r="2594"/>
+    <row r="2595"/>
     <row r="2596">
       <c r="A2596" t="inlineStr">
         <is>
@@ -27403,6 +27597,8 @@
         <v/>
       </c>
     </row>
+    <row r="2600"/>
+    <row r="2601"/>
     <row r="2602">
       <c r="A2602" t="inlineStr">
         <is>
@@ -27482,6 +27678,7 @@
         <v/>
       </c>
     </row>
+    <row r="2609"/>
     <row r="2610">
       <c r="A2610" t="inlineStr">
         <is>
@@ -27535,6 +27732,7 @@
         <v/>
       </c>
     </row>
+    <row r="2614"/>
     <row r="2615">
       <c r="A2615" t="inlineStr">
         <is>
@@ -27595,6 +27793,8 @@
         <v/>
       </c>
     </row>
+    <row r="2620"/>
+    <row r="2621"/>
     <row r="2622">
       <c r="A2622" t="inlineStr">
         <is>
@@ -27680,6 +27880,7 @@
         <v/>
       </c>
     </row>
+    <row r="2630"/>
     <row r="2631">
       <c r="A2631" t="inlineStr">
         <is>
@@ -27733,6 +27934,8 @@
         <v/>
       </c>
     </row>
+    <row r="2635"/>
+    <row r="2636"/>
     <row r="2637">
       <c r="A2637" t="inlineStr">
         <is>
@@ -27797,6 +28000,8 @@
         <v/>
       </c>
     </row>
+    <row r="2643"/>
+    <row r="2644"/>
     <row r="2645">
       <c r="A2645" t="inlineStr">
         <is>
@@ -27855,6 +28060,7 @@
         <v/>
       </c>
     </row>
+    <row r="2650"/>
     <row r="2651">
       <c r="A2651" t="inlineStr">
         <is>
@@ -27908,6 +28114,7 @@
         <v/>
       </c>
     </row>
+    <row r="2655"/>
     <row r="2656">
       <c r="A2656" t="inlineStr">
         <is>
@@ -28028,6 +28235,148 @@
       <c r="C2664">
         <f>C2663/ABS(C2657+C2658+C2659)</f>
         <v/>
+      </c>
+    </row>
+    <row r="2665"/>
+    <row r="2666"/>
+    <row r="2667">
+      <c r="A2667" t="inlineStr">
+        <is>
+          <t>2026.10.22</t>
+        </is>
+      </c>
+      <c r="B2667" t="n">
+        <v>2152796.55</v>
+      </c>
+      <c r="C2667" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2668">
+      <c r="A2668" t="n">
+        <v>-76314.16</v>
+      </c>
+      <c r="B2668">
+        <f>+B2667+A2668</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2669">
+      <c r="A2669" t="n">
+        <v>-76419.99000000001</v>
+      </c>
+      <c r="B2669">
+        <f>+B2668+A2669</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2670">
+      <c r="A2670" t="n">
+        <v>-76209</v>
+      </c>
+      <c r="B2670">
+        <f>+B2669+A2670</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2671">
+      <c r="A2671" t="n">
+        <v>-76180.5</v>
+      </c>
+      <c r="B2671">
+        <f>+B2670+A2671</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2672">
+      <c r="B2672" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2672" s="80">
+        <f>SUM(C2668:C2671)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2673">
+      <c r="B2673" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2673" s="80">
+        <f>+B2671-B2667-A2668-A2669-A2670-A2671</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2675">
+      <c r="A2675" t="inlineStr">
+        <is>
+          <t>累積留倉   400股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2676">
+      <c r="A2676" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2676" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2676" t="n">
+        <v>-76314.16</v>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2677" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2677" t="n">
+        <v>-76419.99000000001</v>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="A2678" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2678" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2678" t="n">
+        <v>-76209</v>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="A2679" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2679" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2679" t="n">
+        <v>-76180.5</v>
       </c>
     </row>
   </sheetData>
@@ -28042,7 +28391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -28916,6 +29265,18 @@
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="86" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B73" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73">
+        <f>C72+B73</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502: 加碼留倉範本 + trades-only 已寫入日不擋 gate + 畫面還原前景 + Boss patch 20261028
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2679"/>
+  <dimension ref="A1:E2710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -28312,71 +28312,394 @@
         <v/>
       </c>
     </row>
-    <row r="2675">
-      <c r="A2675" t="inlineStr">
-        <is>
-          <t>累積留倉   400股</t>
-        </is>
-      </c>
-    </row>
+    <row r="2674"/>
+    <row r="2675"/>
     <row r="2676">
       <c r="A2676" t="inlineStr">
         <is>
+          <t>2026.10.23</t>
+        </is>
+      </c>
+      <c r="B2676" t="n">
+        <v>2078463.01</v>
+      </c>
+      <c r="C2676" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" t="n">
+        <v>-76087</v>
+      </c>
+      <c r="B2677">
+        <f>+B2676+A2677</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="B2678" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2678" s="80">
+        <f>SUM(C2677:C2677)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="B2679" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2679" s="80">
+        <f>+B2677-B2676-A2677</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2680"/>
+    <row r="2681"/>
+    <row r="2682">
+      <c r="A2682" t="inlineStr">
+        <is>
+          <t>2026.10.27</t>
+        </is>
+      </c>
+      <c r="B2682" t="n">
+        <v>2002376.01</v>
+      </c>
+      <c r="C2682" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+    </row>
+    <row r="2683">
+      <c r="A2683" t="n">
+        <v>-76636</v>
+      </c>
+      <c r="B2683">
+        <f>+B2682+A2683</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2684">
+      <c r="A2684" t="n">
+        <v>76749.96000000001</v>
+      </c>
+      <c r="B2684">
+        <f>+B2683+A2684</f>
+        <v/>
+      </c>
+      <c r="C2684" t="n">
+        <v>113.96</v>
+      </c>
+    </row>
+    <row r="2685">
+      <c r="A2685" t="n">
+        <v>77035.91</v>
+      </c>
+      <c r="B2685">
+        <f>+B2684+A2685</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2686">
+      <c r="A2686" t="n">
+        <v>77030.91</v>
+      </c>
+      <c r="B2686">
+        <f>+B2685+A2686</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2687">
+      <c r="A2687" t="n">
+        <v>77034.24000000001</v>
+      </c>
+      <c r="B2687">
+        <f>+B2686+A2687</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2688">
+      <c r="A2688" t="n">
+        <v>77041.08</v>
+      </c>
+      <c r="B2688">
+        <f>+B2687+A2688</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2689">
+      <c r="A2689" t="n">
+        <v>77043.41</v>
+      </c>
+      <c r="B2689">
+        <f>+B2688+A2689</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2690">
+      <c r="B2690" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2690" s="80">
+        <f>SUM(C2683:C2689)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2691">
+      <c r="B2691" t="inlineStr">
+        <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2691" s="80">
+        <f>+B2689-B2682-A2685-A2686-A2687-A2688-A2689</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2693">
+      <c r="A2693" t="inlineStr">
+        <is>
+          <t>2026.10.27當沖</t>
+        </is>
+      </c>
+      <c r="B2693" t="inlineStr">
+        <is>
+          <t>買</t>
+        </is>
+      </c>
+      <c r="C2693" s="80">
+        <f>SUMIF(A2683:A2684,"&lt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2694">
+      <c r="A2694">
+        <f>"SPY " &amp; COUNT(C2683:C2684) * 100 &amp; "股"</f>
+        <v/>
+      </c>
+      <c r="B2694" t="inlineStr">
+        <is>
+          <t>賣</t>
+        </is>
+      </c>
+      <c r="C2694" s="80">
+        <f>SUMIF(A2683:A2684,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2695">
+      <c r="B2695" t="inlineStr">
+        <is>
+          <t>當日損益</t>
+        </is>
+      </c>
+      <c r="C2695" s="80">
+        <f>+C2693+C2694</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2696">
+      <c r="B2696" t="inlineStr">
+        <is>
+          <t>當日損益 %</t>
+        </is>
+      </c>
+      <c r="C2696" s="45">
+        <f>C2695/ABS(C2693)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2698">
+      <c r="A2698" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2699">
+      <c r="A2699" t="inlineStr">
+        <is>
           <t>2026.10.22 留倉</t>
         </is>
       </c>
-      <c r="B2676" t="inlineStr">
+      <c r="B2699" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2676" t="n">
+      <c r="C2699" t="n">
         <v>-76314.16</v>
       </c>
     </row>
-    <row r="2677">
-      <c r="A2677" t="inlineStr">
+    <row r="2700">
+      <c r="A2700" t="inlineStr">
         <is>
           <t>2026.10.22 留倉</t>
         </is>
       </c>
-      <c r="B2677" t="inlineStr">
+      <c r="B2700" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2677" t="n">
+      <c r="C2700" t="n">
         <v>-76419.99000000001</v>
       </c>
     </row>
-    <row r="2678">
-      <c r="A2678" t="inlineStr">
+    <row r="2701">
+      <c r="A2701" t="inlineStr">
         <is>
           <t>2026.10.22 留倉</t>
         </is>
       </c>
-      <c r="B2678" t="inlineStr">
+      <c r="B2701" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2678" t="n">
+      <c r="C2701" t="n">
         <v>-76209</v>
       </c>
     </row>
-    <row r="2679">
-      <c r="A2679" t="inlineStr">
+    <row r="2702">
+      <c r="A2702" t="inlineStr">
         <is>
           <t>2026.10.22 留倉</t>
         </is>
       </c>
-      <c r="B2679" t="inlineStr">
+      <c r="B2702" t="inlineStr">
         <is>
           <t>買 100股</t>
         </is>
       </c>
-      <c r="C2679" t="n">
+      <c r="C2702" t="n">
         <v>-76180.5</v>
+      </c>
+    </row>
+    <row r="2703">
+      <c r="A2703" t="inlineStr">
+        <is>
+          <t>2026.10.23 留倉</t>
+        </is>
+      </c>
+      <c r="B2703" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2703" t="n">
+        <v>-76087</v>
+      </c>
+    </row>
+    <row r="2704">
+      <c r="A2704" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2704" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2704">
+        <f>+A2689</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2705">
+      <c r="A2705" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2705" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2705">
+        <f>+A2688</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2706">
+      <c r="A2706" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2706" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2706">
+        <f>+A2687</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2707">
+      <c r="A2707" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2707" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2707">
+        <f>+A2686</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2708">
+      <c r="A2708" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2708" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2708">
+        <f>+A2685</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2709">
+      <c r="B2709" t="inlineStr">
+        <is>
+          <t>平倉損益</t>
+        </is>
+      </c>
+      <c r="C2709">
+        <f>C2699+C2700+C2701+C2702+C2703+C2704+C2705+C2706+C2707+C2708</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2710">
+      <c r="B2710" t="inlineStr">
+        <is>
+          <t>平倉損益 %</t>
+        </is>
+      </c>
+      <c r="C2710">
+        <f>C2709/ABS(C2699+C2700+C2701+C2702+C2703)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -28391,7 +28714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -29277,6 +29600,30 @@
         <v/>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="86" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B74" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74">
+        <f>C73+B74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="86" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B75" t="n">
+        <v>4088.86</v>
+      </c>
+      <c r="C75">
+        <f>C74+B75</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-30 12:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2710"/>
+  <dimension ref="A1:E2722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -28465,6 +28465,7 @@
         <v/>
       </c>
     </row>
+    <row r="2692"/>
     <row r="2693">
       <c r="A2693" t="inlineStr">
         <is>
@@ -28518,187 +28519,301 @@
         <v/>
       </c>
     </row>
-    <row r="2698">
-      <c r="A2698" t="inlineStr">
-        <is>
-          <t>累積留倉   0股</t>
-        </is>
-      </c>
-    </row>
+    <row r="2697"/>
+    <row r="2698"/>
     <row r="2699">
       <c r="A2699" t="inlineStr">
         <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2699" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2699" t="n">
-        <v>-76314.16</v>
+          <t>2026.10.29</t>
+        </is>
+      </c>
+      <c r="B2699" t="n">
+        <v>2387675.52</v>
+      </c>
+      <c r="C2699" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
       </c>
     </row>
     <row r="2700">
-      <c r="A2700" t="inlineStr">
-        <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2700" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2700" t="n">
-        <v>-76419.99000000001</v>
+      <c r="A2700" t="n">
+        <v>-76829</v>
+      </c>
+      <c r="B2700">
+        <f>+B2699+A2700</f>
+        <v/>
       </c>
     </row>
     <row r="2701">
-      <c r="A2701" t="inlineStr">
-        <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2701" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
+      <c r="A2701" t="n">
+        <v>76885.99000000001</v>
+      </c>
+      <c r="B2701">
+        <f>+B2700+A2701</f>
+        <v/>
       </c>
       <c r="C2701" t="n">
-        <v>-76209</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="2702">
-      <c r="A2702" t="inlineStr">
-        <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
       <c r="B2702" t="inlineStr">
         <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2702" t="n">
-        <v>-76180.5</v>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2702" s="80">
+        <f>SUM(C2700:C2701)</f>
+        <v/>
       </c>
     </row>
     <row r="2703">
-      <c r="A2703" t="inlineStr">
-        <is>
-          <t>2026.10.23 留倉</t>
-        </is>
-      </c>
       <c r="B2703" t="inlineStr">
         <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2703" t="n">
-        <v>-76087</v>
-      </c>
-    </row>
-    <row r="2704">
-      <c r="A2704" t="inlineStr">
-        <is>
-          <t>2026.10.27 平倉</t>
-        </is>
-      </c>
-      <c r="B2704" t="inlineStr">
-        <is>
-          <t>賣100股</t>
-        </is>
-      </c>
-      <c r="C2704">
-        <f>+A2689</f>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2703" s="80">
+        <f>+B2701-B2699</f>
         <v/>
       </c>
     </row>
     <row r="2705">
       <c r="A2705" t="inlineStr">
         <is>
+          <t>2026.10.29當沖</t>
+        </is>
+      </c>
+      <c r="B2705" t="inlineStr">
+        <is>
+          <t>買</t>
+        </is>
+      </c>
+      <c r="C2705" s="80">
+        <f>SUMIF(A2700:A2701,"&lt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2706">
+      <c r="A2706">
+        <f>"SPY " &amp; COUNT(C2700:C2701) * 100 &amp; "股"</f>
+        <v/>
+      </c>
+      <c r="B2706" t="inlineStr">
+        <is>
+          <t>賣</t>
+        </is>
+      </c>
+      <c r="C2706" s="80">
+        <f>SUMIF(A2700:A2701,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2707">
+      <c r="B2707" t="inlineStr">
+        <is>
+          <t>當日損益</t>
+        </is>
+      </c>
+      <c r="C2707" s="80">
+        <f>+C2705+C2706</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2708">
+      <c r="B2708" t="inlineStr">
+        <is>
+          <t>當日損益 %</t>
+        </is>
+      </c>
+      <c r="C2708" s="45">
+        <f>C2707/ABS(C2705)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2709"/>
+    <row r="2710">
+      <c r="A2710" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2711">
+      <c r="A2711" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2711" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2711" t="n">
+        <v>-76314.16</v>
+      </c>
+    </row>
+    <row r="2712">
+      <c r="A2712" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2712" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2712" t="n">
+        <v>-76419.99000000001</v>
+      </c>
+    </row>
+    <row r="2713">
+      <c r="A2713" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2713" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2713" t="n">
+        <v>-76209</v>
+      </c>
+    </row>
+    <row r="2714">
+      <c r="A2714" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2714" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2714" t="n">
+        <v>-76180.5</v>
+      </c>
+    </row>
+    <row r="2715">
+      <c r="A2715" t="inlineStr">
+        <is>
+          <t>2026.10.23 留倉</t>
+        </is>
+      </c>
+      <c r="B2715" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2715" t="n">
+        <v>-76087</v>
+      </c>
+    </row>
+    <row r="2716">
+      <c r="A2716" t="inlineStr">
+        <is>
           <t>2026.10.27 平倉</t>
         </is>
       </c>
-      <c r="B2705" t="inlineStr">
+      <c r="B2716" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2705">
+      <c r="C2716">
+        <f>+A2689</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2717">
+      <c r="A2717" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2717" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2717">
         <f>+A2688</f>
         <v/>
       </c>
     </row>
-    <row r="2706">
-      <c r="A2706" t="inlineStr">
+    <row r="2718">
+      <c r="A2718" t="inlineStr">
         <is>
           <t>2026.10.27 平倉</t>
         </is>
       </c>
-      <c r="B2706" t="inlineStr">
+      <c r="B2718" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2706">
+      <c r="C2718">
         <f>+A2687</f>
         <v/>
       </c>
     </row>
-    <row r="2707">
-      <c r="A2707" t="inlineStr">
+    <row r="2719">
+      <c r="A2719" t="inlineStr">
         <is>
           <t>2026.10.27 平倉</t>
         </is>
       </c>
-      <c r="B2707" t="inlineStr">
+      <c r="B2719" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2707">
+      <c r="C2719">
         <f>+A2686</f>
         <v/>
       </c>
     </row>
-    <row r="2708">
-      <c r="A2708" t="inlineStr">
+    <row r="2720">
+      <c r="A2720" t="inlineStr">
         <is>
           <t>2026.10.27 平倉</t>
         </is>
       </c>
-      <c r="B2708" t="inlineStr">
+      <c r="B2720" t="inlineStr">
         <is>
           <t>賣100股</t>
         </is>
       </c>
-      <c r="C2708">
+      <c r="C2720">
         <f>+A2685</f>
         <v/>
       </c>
     </row>
-    <row r="2709">
-      <c r="B2709" t="inlineStr">
+    <row r="2721">
+      <c r="B2721" t="inlineStr">
         <is>
           <t>平倉損益</t>
         </is>
       </c>
-      <c r="C2709">
-        <f>C2699+C2700+C2701+C2702+C2703+C2704+C2705+C2706+C2707+C2708</f>
-        <v/>
-      </c>
-    </row>
-    <row r="2710">
-      <c r="B2710" t="inlineStr">
+      <c r="C2721">
+        <f>C2711+C2712+C2713+C2714+C2715+C2716+C2717+C2718+C2719+C2720</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2722">
+      <c r="B2722" t="inlineStr">
         <is>
           <t>平倉損益 %</t>
         </is>
       </c>
-      <c r="C2710">
-        <f>C2709/ABS(C2699+C2700+C2701+C2702+C2703)</f>
+      <c r="C2722">
+        <f>C2721/ABS(C2711+C2712+C2713+C2714+C2715)</f>
         <v/>
       </c>
     </row>
@@ -28714,7 +28829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -29624,6 +29739,18 @@
         <v/>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="86" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B76" t="n">
+        <v>56.99</v>
+      </c>
+      <c r="C76">
+        <f>C75+B76</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
p502 sync 2026-10-31 10:00
</commit_message>
<xml_diff>
--- a/CS交易紀錄.xlsx
+++ b/CS交易紀錄.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="170" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -131,6 +131,10 @@
       <color rgb="FFFF0000"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
     </font>
   </fonts>
   <fills count="12">
@@ -255,7 +259,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -478,6 +482,7 @@
     </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -848,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2722"/>
+  <dimension ref="A1:D2735"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.875" customWidth="1" style="44" min="1" max="1"/>
@@ -28579,6 +28584,7 @@
         <v/>
       </c>
     </row>
+    <row r="2704"/>
     <row r="2705">
       <c r="A2705" t="inlineStr">
         <is>
@@ -28632,188 +28638,312 @@
         <v/>
       </c>
     </row>
-    <row r="2709"/>
-    <row r="2710">
-      <c r="A2710" t="inlineStr">
-        <is>
-          <t>累積留倉   0股</t>
-        </is>
-      </c>
-    </row>
     <row r="2711">
       <c r="A2711" t="inlineStr">
         <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2711" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2711" t="n">
-        <v>-76314.16</v>
+          <t>2026.10.30</t>
+        </is>
+      </c>
+      <c r="B2711" t="n">
+        <v>2387675.52</v>
+      </c>
+      <c r="C2711" t="inlineStr">
+        <is>
+          <t>損益</t>
+        </is>
+      </c>
+      <c r="D2711" s="90" t="inlineStr">
+        <is>
+          <t>⚠️待修正：非交易現金異動 10/30 16:25 TYPE=DOI AMOUNT=2077.72 (STATE STREET SPDR S&amp;P 500 ETF TRUST 2077) — 需人工判斷是否入金/出金；非交易現金異動 10/30 16:25 TYPE=JRN AMOUNT=-623.32 (STATE STREET SPDR S&amp;P 500 ETF TRUST -623) — 需人工判斷是否入金/出金；BALANCE 對不上 @ 10/30 21:41:22 ref=1008493673759: 重建=2311593.30 vs 對帳單=2313047.70 差=-1454.40；BALANCE 對不上 @ 10/30 21:53:59 ref=1008494629631: 重建=2235546.32 vs 對帳單=2237000.72 差=-1454.40；BALANCE 對不上 @ 10/30 22:09:23 ref=1008495481841: 重建=2159565.33 vs 對帳單=2161019.73 差=-1454.40；BALANCE 對不上 @ 10/30 22:12:09 ref=1008496306250: 重建=2083659.34 vs 對帳單=2085113.74 差=-1454.40；BALANCE 對不上 @ 10/30 22:13:03 ref=1008496306376: 重建=2007778.84 vs 對帳單=2009233.24 差=-1454.40；BALANCE 對不上 @ 10/30 23:16:12 ref=1008499335110: 重建=1931913.34 vs 對帳單=1933367.74 差=-1454.40；⚠️需人工確認：Σcol1(-455762.18) ≠ 收-開(-454307.78)，差 -1454.40</t>
+        </is>
       </c>
     </row>
     <row r="2712">
-      <c r="A2712" t="inlineStr">
-        <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2712" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2712" t="n">
-        <v>-76419.99000000001</v>
+      <c r="A2712" t="n">
+        <v>2077.72</v>
+      </c>
+      <c r="B2712">
+        <f>+B2711+A2712</f>
+        <v/>
+      </c>
+      <c r="D2712" t="inlineStr">
+        <is>
+          <t>DOI STATE STREET SPDR S&amp;P 500 ETF TRUST 2077</t>
+        </is>
       </c>
     </row>
     <row r="2713">
-      <c r="A2713" t="inlineStr">
-        <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2713" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2713" t="n">
-        <v>-76209</v>
+      <c r="A2713" t="n">
+        <v>-623.3200000000001</v>
+      </c>
+      <c r="B2713">
+        <f>+B2712+A2713</f>
+        <v/>
+      </c>
+      <c r="D2713" t="inlineStr">
+        <is>
+          <t>JRN STATE STREET SPDR S&amp;P 500 ETF TRUST -623</t>
+        </is>
       </c>
     </row>
     <row r="2714">
-      <c r="A2714" t="inlineStr">
-        <is>
-          <t>2026.10.22 留倉</t>
-        </is>
-      </c>
-      <c r="B2714" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2714" t="n">
-        <v>-76180.5</v>
+      <c r="A2714" t="n">
+        <v>-76082.22</v>
+      </c>
+      <c r="B2714">
+        <f>+B2713+A2714</f>
+        <v/>
       </c>
     </row>
     <row r="2715">
-      <c r="A2715" t="inlineStr">
-        <is>
-          <t>2026.10.23 留倉</t>
-        </is>
-      </c>
-      <c r="B2715" t="inlineStr">
-        <is>
-          <t>買 100股</t>
-        </is>
-      </c>
-      <c r="C2715" t="n">
-        <v>-76087</v>
+      <c r="A2715" t="n">
+        <v>-76046.98</v>
+      </c>
+      <c r="B2715">
+        <f>+B2714+A2715</f>
+        <v/>
       </c>
     </row>
     <row r="2716">
-      <c r="A2716" t="inlineStr">
-        <is>
-          <t>2026.10.27 平倉</t>
-        </is>
-      </c>
-      <c r="B2716" t="inlineStr">
-        <is>
-          <t>賣100股</t>
-        </is>
-      </c>
-      <c r="C2716">
-        <f>+A2689</f>
+      <c r="A2716" t="n">
+        <v>-75980.99000000001</v>
+      </c>
+      <c r="B2716">
+        <f>+B2715+A2716</f>
         <v/>
       </c>
     </row>
     <row r="2717">
-      <c r="A2717" t="inlineStr">
-        <is>
-          <t>2026.10.27 平倉</t>
-        </is>
-      </c>
-      <c r="B2717" t="inlineStr">
-        <is>
-          <t>賣100股</t>
-        </is>
-      </c>
-      <c r="C2717">
-        <f>+A2688</f>
+      <c r="A2717" t="n">
+        <v>-75905.99000000001</v>
+      </c>
+      <c r="B2717">
+        <f>+B2716+A2717</f>
         <v/>
       </c>
     </row>
     <row r="2718">
-      <c r="A2718" t="inlineStr">
-        <is>
-          <t>2026.10.27 平倉</t>
-        </is>
-      </c>
-      <c r="B2718" t="inlineStr">
-        <is>
-          <t>賣100股</t>
-        </is>
-      </c>
-      <c r="C2718">
-        <f>+A2687</f>
+      <c r="A2718" t="n">
+        <v>-75880.5</v>
+      </c>
+      <c r="B2718">
+        <f>+B2717+A2718</f>
         <v/>
       </c>
     </row>
     <row r="2719">
-      <c r="A2719" t="inlineStr">
-        <is>
-          <t>2026.10.27 平倉</t>
-        </is>
-      </c>
-      <c r="B2719" t="inlineStr">
-        <is>
-          <t>賣100股</t>
-        </is>
-      </c>
-      <c r="C2719">
-        <f>+A2686</f>
+      <c r="A2719" t="n">
+        <v>-75865.5</v>
+      </c>
+      <c r="B2719">
+        <f>+B2718+A2719</f>
         <v/>
       </c>
     </row>
     <row r="2720">
-      <c r="A2720" t="inlineStr">
-        <is>
-          <t>2026.10.27 平倉</t>
-        </is>
-      </c>
       <c r="B2720" t="inlineStr">
         <is>
-          <t>賣100股</t>
-        </is>
-      </c>
-      <c r="C2720">
-        <f>+A2685</f>
+          <t xml:space="preserve">合計 </t>
+        </is>
+      </c>
+      <c r="C2720" s="80">
+        <f>SUM(C2712:C2719)</f>
         <v/>
       </c>
     </row>
     <row r="2721">
       <c r="B2721" t="inlineStr">
         <is>
+          <t>核驗</t>
+        </is>
+      </c>
+      <c r="C2721" s="80">
+        <f>+B2719-B2711</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2722"/>
+    <row r="2723">
+      <c r="A2723" t="inlineStr">
+        <is>
+          <t>累積留倉   0股</t>
+        </is>
+      </c>
+    </row>
+    <row r="2724">
+      <c r="A2724" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2724" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2724" t="n">
+        <v>-76314.16</v>
+      </c>
+    </row>
+    <row r="2725">
+      <c r="A2725" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2725" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2725" t="n">
+        <v>-76419.99000000001</v>
+      </c>
+    </row>
+    <row r="2726">
+      <c r="A2726" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2726" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2726" t="n">
+        <v>-76209</v>
+      </c>
+    </row>
+    <row r="2727">
+      <c r="A2727" t="inlineStr">
+        <is>
+          <t>2026.10.22 留倉</t>
+        </is>
+      </c>
+      <c r="B2727" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2727" t="n">
+        <v>-76180.5</v>
+      </c>
+    </row>
+    <row r="2728">
+      <c r="A2728" t="inlineStr">
+        <is>
+          <t>2026.10.23 留倉</t>
+        </is>
+      </c>
+      <c r="B2728" t="inlineStr">
+        <is>
+          <t>買 100股</t>
+        </is>
+      </c>
+      <c r="C2728" t="n">
+        <v>-76087</v>
+      </c>
+    </row>
+    <row r="2729">
+      <c r="A2729" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2729" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2729">
+        <f>+A2689</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2730">
+      <c r="A2730" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2730" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2730">
+        <f>+A2688</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2731">
+      <c r="A2731" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2731" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2731">
+        <f>+A2687</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2732">
+      <c r="A2732" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2732" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2732">
+        <f>+A2686</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2733">
+      <c r="A2733" t="inlineStr">
+        <is>
+          <t>2026.10.27 平倉</t>
+        </is>
+      </c>
+      <c r="B2733" t="inlineStr">
+        <is>
+          <t>賣100股</t>
+        </is>
+      </c>
+      <c r="C2733">
+        <f>+A2685</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2734">
+      <c r="B2734" t="inlineStr">
+        <is>
           <t>平倉損益</t>
         </is>
       </c>
-      <c r="C2721">
-        <f>C2711+C2712+C2713+C2714+C2715+C2716+C2717+C2718+C2719+C2720</f>
-        <v/>
-      </c>
-    </row>
-    <row r="2722">
-      <c r="B2722" t="inlineStr">
+      <c r="C2734">
+        <f>C2724+C2725+C2726+C2727+C2728+C2729+C2730+C2731+C2732+C2733</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2735">
+      <c r="B2735" t="inlineStr">
         <is>
           <t>平倉損益 %</t>
         </is>
       </c>
-      <c r="C2722">
-        <f>C2721/ABS(C2711+C2712+C2713+C2714+C2715)</f>
+      <c r="C2735">
+        <f>C2734/ABS(C2724+C2725+C2726+C2727+C2728)</f>
         <v/>
       </c>
     </row>
@@ -28829,7 +28959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="18.75" customWidth="1" style="44" min="1" max="1"/>
@@ -29751,6 +29881,18 @@
         <v/>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="86" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B77" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77">
+        <f>C76+B77</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>